<commit_message>
Excel data day 2
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D900F89C-B28D-40DA-8156-408657CF9D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7258DE0-75E8-4876-9EC8-4EB7B33D817F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -215,6 +215,12 @@
   </si>
   <si>
     <t>Felt extremely tired after today's classes</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>I had cold today so being in class was tough.</t>
   </si>
 </sst>
 </file>
@@ -1056,7 +1062,7 @@
         <v>17</v>
       </c>
       <c r="F7" s="14">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G7" s="14">
         <v>6</v>
@@ -1066,11 +1072,11 @@
       </c>
       <c r="I7" s="15">
         <f t="shared" si="0"/>
-        <v>815</v>
+        <v>715</v>
       </c>
       <c r="J7" s="15">
         <f t="shared" si="1"/>
-        <v>625</v>
+        <v>725</v>
       </c>
       <c r="K7" s="16" t="s">
         <v>57</v>
@@ -1085,27 +1091,51 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+    <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="13">
+        <v>46253</v>
+      </c>
+      <c r="B8" s="14">
+        <v>390</v>
+      </c>
+      <c r="C8" s="14">
+        <v>18</v>
+      </c>
+      <c r="D8" s="14">
+        <v>25</v>
+      </c>
+      <c r="E8" s="14">
+        <v>70</v>
+      </c>
+      <c r="F8" s="14">
+        <v>350</v>
+      </c>
+      <c r="G8" s="14">
+        <v>7</v>
+      </c>
+      <c r="H8" s="14">
+        <v>60</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>913</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
+        <v>527</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="13"/>

</xml_diff>

<commit_message>
Updated Excel Data Day 3
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7258DE0-75E8-4876-9EC8-4EB7B33D817F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364605AE-6D4E-4052-942E-81C3E8042FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -221,6 +221,9 @@
   </si>
   <si>
     <t>I had cold today so being in class was tough.</t>
+  </si>
+  <si>
+    <t>Didn't attend my last class because of my fever.</t>
   </si>
 </sst>
 </file>
@@ -1137,27 +1140,51 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14"/>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="str">
+    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="13">
+        <v>46254</v>
+      </c>
+      <c r="B9" s="14">
+        <v>370</v>
+      </c>
+      <c r="C9" s="14">
+        <v>45</v>
+      </c>
+      <c r="D9" s="14">
+        <v>40</v>
+      </c>
+      <c r="E9" s="14">
+        <v>55</v>
+      </c>
+      <c r="F9" s="14">
+        <v>150</v>
+      </c>
+      <c r="G9" s="14">
+        <v>3</v>
+      </c>
+      <c r="H9" s="14">
+        <v>55</v>
+      </c>
+      <c r="I9" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="15" t="str">
+        <v>715</v>
+      </c>
+      <c r="J9" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="17"/>
+        <v>725</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="L9" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M9" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>

</xml_diff>

<commit_message>
Excel data updated Day 4
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364605AE-6D4E-4052-942E-81C3E8042FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77AF795F-D0E3-4FBA-9506-A66973889089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -224,6 +224,9 @@
   </si>
   <si>
     <t>Didn't attend my last class because of my fever.</t>
+  </si>
+  <si>
+    <t>Didn't attend any lecture due to punjab being closed</t>
   </si>
 </sst>
 </file>
@@ -1186,27 +1189,51 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="15" t="str">
+    <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="13">
+        <v>46255</v>
+      </c>
+      <c r="B10" s="14">
+        <v>440</v>
+      </c>
+      <c r="C10" s="14">
+        <v>15</v>
+      </c>
+      <c r="D10" s="14">
+        <v>70</v>
+      </c>
+      <c r="E10" s="14">
+        <v>95</v>
+      </c>
+      <c r="F10" s="14">
+        <v>0</v>
+      </c>
+      <c r="G10" s="14">
+        <v>0</v>
+      </c>
+      <c r="H10" s="14">
+        <v>120</v>
+      </c>
+      <c r="I10" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="15" t="str">
+        <v>740</v>
+      </c>
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="17"/>
+        <v>700</v>
+      </c>
+      <c r="K10" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L10" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M10" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="13"/>

</xml_diff>

<commit_message>
Updated Excel Data Day 5
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E050D36-9A4D-4223-93DE-2412A85B2BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E763953-15B6-4FCF-BA4F-BAA36E3CA69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -229,7 +229,7 @@
     <t>Didn't attend any lecture due to punjab being closed</t>
   </si>
   <si>
-    <t>Monday is added for our timetable so worry and stress</t>
+    <t>Monday is added to our timetable so less time for study.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updated Excel Data Day 6
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E763953-15B6-4FCF-BA4F-BAA36E3CA69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCD1D0D-7772-4335-B875-A6B53815D23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -230,6 +230,12 @@
   </si>
   <si>
     <t>Monday is added to our timetable so less time for study.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Today is Sunday so class is off. Ready for Monday's Class</t>
   </si>
 </sst>
 </file>
@@ -1284,27 +1290,51 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+    <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B12" s="14">
+        <v>540</v>
+      </c>
+      <c r="C12" s="14">
+        <v>20</v>
+      </c>
+      <c r="D12" s="14">
+        <v>80</v>
+      </c>
+      <c r="E12" s="14">
+        <v>100</v>
+      </c>
+      <c r="F12" s="14">
+        <v>0</v>
+      </c>
+      <c r="G12" s="14">
+        <v>0</v>
+      </c>
+      <c r="H12" s="14">
+        <v>90</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>610</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="13"/>

</xml_diff>

<commit_message>
Update Excel Data Day 7
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBCD1D0D-7772-4335-B875-A6B53815D23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{034337C7-3DEA-42F5-A373-464BEF3EEFA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Today is Sunday so class is off. Ready for Monday's Class</t>
+  </si>
+  <si>
+    <t>Today I was in Advance communication class feeling lonely and nervous</t>
   </si>
 </sst>
 </file>
@@ -1336,27 +1339,51 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+    <row r="13" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B13" s="14">
+        <v>370</v>
+      </c>
+      <c r="C13" s="14">
+        <v>10</v>
+      </c>
+      <c r="D13" s="14">
+        <v>20</v>
+      </c>
+      <c r="E13" s="14">
+        <v>60</v>
+      </c>
+      <c r="F13" s="14">
+        <v>200</v>
+      </c>
+      <c r="G13" s="14">
+        <v>4</v>
+      </c>
+      <c r="H13" s="14">
+        <v>80</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>740</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>700</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>

</xml_diff>

<commit_message>
Updated Excel Data Day 11
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5D2270B-41D6-445A-B498-0B1D7EA985A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294D1D48-5CFD-4052-8CA3-3B0446DB37C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="74">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -249,6 +249,15 @@
   <si>
     <t>Sr. No.</t>
   </si>
+  <si>
+    <t>Stressed</t>
+  </si>
+  <si>
+    <t>Very Unsatisfied</t>
+  </si>
+  <si>
+    <t>I am not getting time to work on myself. I have to change myself.</t>
+  </si>
 </sst>
 </file>
 
@@ -379,7 +388,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -408,9 +417,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1012,7 +1018,7 @@
       </c>
     </row>
     <row r="6" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="16">
+      <c r="A6" s="11">
         <f>IF(B6&lt;&gt;"",COUNT($B$6:B6),"")</f>
         <v>1</v>
       </c>
@@ -1062,7 +1068,7 @@
       </c>
     </row>
     <row r="7" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A7" s="16">
+      <c r="A7" s="11">
         <f>IF(B7&lt;&gt;"",COUNT($B$6:B7),"")</f>
         <v>2</v>
       </c>
@@ -1112,7 +1118,7 @@
       </c>
     </row>
     <row r="8" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="16">
+      <c r="A8" s="11">
         <f>IF(B8&lt;&gt;"",COUNT($B$6:B8),"")</f>
         <v>3</v>
       </c>
@@ -1162,7 +1168,7 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="16">
+      <c r="A9" s="11">
         <f>IF(B9&lt;&gt;"",COUNT($B$6:B9),"")</f>
         <v>4</v>
       </c>
@@ -1212,7 +1218,7 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="16">
+      <c r="A10" s="11">
         <f>IF(B10&lt;&gt;"",COUNT($B$6:B10),"")</f>
         <v>5</v>
       </c>
@@ -1262,7 +1268,7 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="16">
+      <c r="A11" s="11">
         <f>IF(B11&lt;&gt;"",COUNT($B$6:B11),"")</f>
         <v>6</v>
       </c>
@@ -1312,7 +1318,7 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="16">
+      <c r="A12" s="11">
         <f>IF(B12&lt;&gt;"",COUNT($B$6:B12),"")</f>
         <v>7</v>
       </c>
@@ -1362,7 +1368,7 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="16">
+      <c r="A13" s="11">
         <f>IF(B13&lt;&gt;"",COUNT($B$6:B13),"")</f>
         <v>8</v>
       </c>
@@ -1412,7 +1418,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="16">
+      <c r="A14" s="11">
         <f>IF(B14&lt;&gt;"",COUNT($B$6:B14),"")</f>
         <v>9</v>
       </c>
@@ -1462,12 +1468,12 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="16">
+      <c r="A15" s="11">
         <f>IF(B15&lt;&gt;"",COUNT($B$6:B15),"")</f>
         <v>10</v>
       </c>
       <c r="B15" s="8">
-        <v>46626</v>
+        <v>46261</v>
       </c>
       <c r="C15" s="9">
         <v>500</v>
@@ -1511,34 +1517,58 @@
         <v>69</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A16" s="16" t="str">
+    <row r="16" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="11">
         <f>IF(B16&lt;&gt;"",COUNT($B$6:B16),"")</f>
-        <v/>
-      </c>
-      <c r="B16" s="8"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="10" t="str">
+        <v>11</v>
+      </c>
+      <c r="B16" s="8">
+        <v>46262</v>
+      </c>
+      <c r="C16" s="9">
+        <v>345</v>
+      </c>
+      <c r="D16" s="9">
+        <v>25</v>
+      </c>
+      <c r="E16" s="9">
+        <v>45</v>
+      </c>
+      <c r="F16" s="9">
+        <v>65</v>
+      </c>
+      <c r="G16" s="9">
+        <v>200</v>
+      </c>
+      <c r="H16" s="9">
+        <v>4</v>
+      </c>
+      <c r="I16" s="9">
+        <v>30</v>
+      </c>
+      <c r="J16" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K16" s="10" t="str">
+        <v>710</v>
+      </c>
+      <c r="K16" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="12"/>
+        <v>730</v>
+      </c>
+      <c r="L16" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="M16" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N16" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O16" s="12" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="str">
+      <c r="A17" s="11" t="str">
         <f>IF(B17&lt;&gt;"",COUNT($B$6:B17),"")</f>
         <v/>
       </c>
@@ -1564,7 +1594,7 @@
       <c r="O17" s="12"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18" s="16" t="str">
+      <c r="A18" s="11" t="str">
         <f>IF(B18&lt;&gt;"",COUNT($B$6:B18),"")</f>
         <v/>
       </c>
@@ -1590,7 +1620,7 @@
       <c r="O18" s="12"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="16" t="str">
+      <c r="A19" s="11" t="str">
         <f>IF(B19&lt;&gt;"",COUNT($B$6:B19),"")</f>
         <v/>
       </c>
@@ -1616,7 +1646,7 @@
       <c r="O19" s="12"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="16" t="str">
+      <c r="A20" s="11" t="str">
         <f>IF(B20&lt;&gt;"",COUNT($B$6:B20),"")</f>
         <v/>
       </c>
@@ -1642,7 +1672,7 @@
       <c r="O20" s="12"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="16" t="str">
+      <c r="A21" s="11" t="str">
         <f>IF(B21&lt;&gt;"",COUNT($B$6:B21),"")</f>
         <v/>
       </c>
@@ -1668,7 +1698,7 @@
       <c r="O21" s="12"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="16" t="str">
+      <c r="A22" s="11" t="str">
         <f>IF(B22&lt;&gt;"",COUNT($B$6:B22),"")</f>
         <v/>
       </c>
@@ -1694,7 +1724,7 @@
       <c r="O22" s="12"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A23" s="16" t="str">
+      <c r="A23" s="11" t="str">
         <f>IF(B23&lt;&gt;"",COUNT($B$6:B23),"")</f>
         <v/>
       </c>
@@ -1720,7 +1750,7 @@
       <c r="O23" s="12"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A24" s="16" t="str">
+      <c r="A24" s="11" t="str">
         <f>IF(B24&lt;&gt;"",COUNT($B$6:B24),"")</f>
         <v/>
       </c>
@@ -1746,7 +1776,7 @@
       <c r="O24" s="12"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A25" s="16" t="str">
+      <c r="A25" s="11" t="str">
         <f>IF(B25&lt;&gt;"",COUNT($B$6:B25),"")</f>
         <v/>
       </c>
@@ -1772,7 +1802,7 @@
       <c r="O25" s="12"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A26" s="16" t="str">
+      <c r="A26" s="11" t="str">
         <f>IF(B26&lt;&gt;"",COUNT($B$6:B26),"")</f>
         <v/>
       </c>
@@ -1798,7 +1828,7 @@
       <c r="O26" s="12"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A27" s="16" t="str">
+      <c r="A27" s="11" t="str">
         <f>IF(B27&lt;&gt;"",COUNT($B$6:B27),"")</f>
         <v/>
       </c>
@@ -1824,7 +1854,7 @@
       <c r="O27" s="12"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A28" s="16" t="str">
+      <c r="A28" s="11" t="str">
         <f>IF(B28&lt;&gt;"",COUNT($B$6:B28),"")</f>
         <v/>
       </c>
@@ -1850,7 +1880,7 @@
       <c r="O28" s="12"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A29" s="16" t="str">
+      <c r="A29" s="11" t="str">
         <f>IF(B29&lt;&gt;"",COUNT($B$6:B29),"")</f>
         <v/>
       </c>
@@ -1876,7 +1906,7 @@
       <c r="O29" s="12"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A30" s="16" t="str">
+      <c r="A30" s="11" t="str">
         <f>IF(B30&lt;&gt;"",COUNT($B$6:B30),"")</f>
         <v/>
       </c>
@@ -1902,7 +1932,7 @@
       <c r="O30" s="12"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A31" s="16" t="str">
+      <c r="A31" s="11" t="str">
         <f>IF(B31&lt;&gt;"",COUNT($B$6:B31),"")</f>
         <v/>
       </c>
@@ -1928,7 +1958,7 @@
       <c r="O31" s="12"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A32" s="16" t="str">
+      <c r="A32" s="11" t="str">
         <f>IF(B32&lt;&gt;"",COUNT($B$6:B32),"")</f>
         <v/>
       </c>
@@ -1954,7 +1984,7 @@
       <c r="O32" s="12"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A33" s="16" t="str">
+      <c r="A33" s="11" t="str">
         <f>IF(B33&lt;&gt;"",COUNT($B$6:B33),"")</f>
         <v/>
       </c>
@@ -1980,7 +2010,7 @@
       <c r="O33" s="12"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A34" s="16" t="str">
+      <c r="A34" s="11" t="str">
         <f>IF(B34&lt;&gt;"",COUNT($B$6:B34),"")</f>
         <v/>
       </c>
@@ -2006,7 +2036,7 @@
       <c r="O34" s="12"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A35" s="16" t="str">
+      <c r="A35" s="11" t="str">
         <f>IF(B35&lt;&gt;"",COUNT($B$6:B35),"")</f>
         <v/>
       </c>
@@ -2032,7 +2062,7 @@
       <c r="O35" s="12"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A36" s="16" t="str">
+      <c r="A36" s="11" t="str">
         <f>IF(B36&lt;&gt;"",COUNT($B$6:B36),"")</f>
         <v/>
       </c>
@@ -2058,7 +2088,7 @@
       <c r="O36" s="12"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A37" s="16" t="str">
+      <c r="A37" s="11" t="str">
         <f>IF(B37&lt;&gt;"",COUNT($B$6:B37),"")</f>
         <v/>
       </c>
@@ -2084,7 +2114,7 @@
       <c r="O37" s="12"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="16" t="str">
+      <c r="A38" s="11" t="str">
         <f>IF(B38&lt;&gt;"",COUNT($B$6:B38),"")</f>
         <v/>
       </c>
@@ -2110,7 +2140,7 @@
       <c r="O38" s="12"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="16" t="str">
+      <c r="A39" s="11" t="str">
         <f>IF(B39&lt;&gt;"",COUNT($B$6:B39),"")</f>
         <v/>
       </c>
@@ -2136,7 +2166,7 @@
       <c r="O39" s="12"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="16" t="str">
+      <c r="A40" s="11" t="str">
         <f>IF(B40&lt;&gt;"",COUNT($B$6:B40),"")</f>
         <v/>
       </c>
@@ -2162,7 +2192,7 @@
       <c r="O40" s="12"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="16" t="str">
+      <c r="A41" s="11" t="str">
         <f>IF(B41&lt;&gt;"",COUNT($B$6:B41),"")</f>
         <v/>
       </c>
@@ -2188,7 +2218,7 @@
       <c r="O41" s="12"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="16" t="str">
+      <c r="A42" s="11" t="str">
         <f>IF(B42&lt;&gt;"",COUNT($B$6:B42),"")</f>
         <v/>
       </c>
@@ -2214,7 +2244,7 @@
       <c r="O42" s="12"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="16" t="str">
+      <c r="A43" s="11" t="str">
         <f>IF(B43&lt;&gt;"",COUNT($B$6:B43),"")</f>
         <v/>
       </c>
@@ -2240,7 +2270,7 @@
       <c r="O43" s="12"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="16" t="str">
+      <c r="A44" s="11" t="str">
         <f>IF(B44&lt;&gt;"",COUNT($B$6:B44),"")</f>
         <v/>
       </c>
@@ -2266,7 +2296,7 @@
       <c r="O44" s="12"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A45" s="16" t="str">
+      <c r="A45" s="11" t="str">
         <f>IF(B45&lt;&gt;"",COUNT($B$6:B45),"")</f>
         <v/>
       </c>
@@ -2292,7 +2322,7 @@
       <c r="O45" s="12"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="16" t="str">
+      <c r="A46" s="11" t="str">
         <f>IF(B46&lt;&gt;"",COUNT($B$6:B46),"")</f>
         <v/>
       </c>
@@ -2318,7 +2348,7 @@
       <c r="O46" s="12"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A47" s="16" t="str">
+      <c r="A47" s="11" t="str">
         <f>IF(B47&lt;&gt;"",COUNT($B$6:B47),"")</f>
         <v/>
       </c>
@@ -2344,7 +2374,7 @@
       <c r="O47" s="12"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A48" s="16" t="str">
+      <c r="A48" s="11" t="str">
         <f>IF(B48&lt;&gt;"",COUNT($B$6:B48),"")</f>
         <v/>
       </c>
@@ -2370,7 +2400,7 @@
       <c r="O48" s="12"/>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="16" t="str">
+      <c r="A49" s="11" t="str">
         <f>IF(B49&lt;&gt;"",COUNT($B$6:B49),"")</f>
         <v/>
       </c>
@@ -2396,7 +2426,7 @@
       <c r="O49" s="12"/>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A50" s="16" t="str">
+      <c r="A50" s="11" t="str">
         <f>IF(B50&lt;&gt;"",COUNT($B$6:B50),"")</f>
         <v/>
       </c>
@@ -2422,7 +2452,7 @@
       <c r="O50" s="12"/>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A51" s="16" t="str">
+      <c r="A51" s="11" t="str">
         <f>IF(B51&lt;&gt;"",COUNT($B$6:B51),"")</f>
         <v/>
       </c>
@@ -2448,7 +2478,7 @@
       <c r="O51" s="12"/>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A52" s="16" t="str">
+      <c r="A52" s="11" t="str">
         <f>IF(B52&lt;&gt;"",COUNT($B$6:B52),"")</f>
         <v/>
       </c>
@@ -2474,7 +2504,7 @@
       <c r="O52" s="12"/>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A53" s="16" t="str">
+      <c r="A53" s="11" t="str">
         <f>IF(B53&lt;&gt;"",COUNT($B$6:B53),"")</f>
         <v/>
       </c>
@@ -2500,7 +2530,7 @@
       <c r="O53" s="12"/>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A54" s="16" t="str">
+      <c r="A54" s="11" t="str">
         <f>IF(B54&lt;&gt;"",COUNT($B$6:B54),"")</f>
         <v/>
       </c>
@@ -2526,7 +2556,7 @@
       <c r="O54" s="12"/>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A55" s="16" t="str">
+      <c r="A55" s="11" t="str">
         <f>IF(B55&lt;&gt;"",COUNT($B$6:B55),"")</f>
         <v/>
       </c>
@@ -2552,7 +2582,7 @@
       <c r="O55" s="12"/>
     </row>
     <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A56" s="16" t="str">
+      <c r="A56" s="11" t="str">
         <f>IF(B56&lt;&gt;"",COUNT($B$6:B56),"")</f>
         <v/>
       </c>
@@ -2578,7 +2608,7 @@
       <c r="O56" s="12"/>
     </row>
     <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A57" s="16" t="str">
+      <c r="A57" s="11" t="str">
         <f>IF(B57&lt;&gt;"",COUNT($B$6:B57),"")</f>
         <v/>
       </c>
@@ -2604,7 +2634,7 @@
       <c r="O57" s="12"/>
     </row>
     <row r="58" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A58" s="16" t="str">
+      <c r="A58" s="11" t="str">
         <f>IF(B58&lt;&gt;"",COUNT($B$6:B58),"")</f>
         <v/>
       </c>
@@ -2630,7 +2660,7 @@
       <c r="O58" s="12"/>
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A59" s="16" t="str">
+      <c r="A59" s="11" t="str">
         <f>IF(B59&lt;&gt;"",COUNT($B$6:B59),"")</f>
         <v/>
       </c>
@@ -2656,7 +2686,7 @@
       <c r="O59" s="12"/>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A60" s="16" t="str">
+      <c r="A60" s="11" t="str">
         <f>IF(B60&lt;&gt;"",COUNT($B$6:B60),"")</f>
         <v/>
       </c>
@@ -2682,7 +2712,7 @@
       <c r="O60" s="12"/>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A61" s="16" t="str">
+      <c r="A61" s="11" t="str">
         <f>IF(B61&lt;&gt;"",COUNT($B$6:B61),"")</f>
         <v/>
       </c>
@@ -2708,7 +2738,7 @@
       <c r="O61" s="12"/>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A62" s="16" t="str">
+      <c r="A62" s="11" t="str">
         <f>IF(B62&lt;&gt;"",COUNT($B$6:B62),"")</f>
         <v/>
       </c>
@@ -2734,7 +2764,7 @@
       <c r="O62" s="12"/>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A63" s="16" t="str">
+      <c r="A63" s="11" t="str">
         <f>IF(B63&lt;&gt;"",COUNT($B$6:B63),"")</f>
         <v/>
       </c>
@@ -2760,7 +2790,7 @@
       <c r="O63" s="12"/>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A64" s="16" t="str">
+      <c r="A64" s="11" t="str">
         <f>IF(B64&lt;&gt;"",COUNT($B$6:B64),"")</f>
         <v/>
       </c>
@@ -2786,7 +2816,7 @@
       <c r="O64" s="12"/>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A65" s="16" t="str">
+      <c r="A65" s="11" t="str">
         <f>IF(B65&lt;&gt;"",COUNT($B$6:B65),"")</f>
         <v/>
       </c>
@@ -2812,7 +2842,7 @@
       <c r="O65" s="12"/>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A66" s="16" t="str">
+      <c r="A66" s="11" t="str">
         <f>IF(B66&lt;&gt;"",COUNT($B$6:B66),"")</f>
         <v/>
       </c>
@@ -2838,7 +2868,7 @@
       <c r="O66" s="12"/>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A67" s="16" t="str">
+      <c r="A67" s="11" t="str">
         <f>IF(B67&lt;&gt;"",COUNT($B$6:B67),"")</f>
         <v/>
       </c>
@@ -2864,7 +2894,7 @@
       <c r="O67" s="12"/>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A68" s="16" t="str">
+      <c r="A68" s="11" t="str">
         <f>IF(B68&lt;&gt;"",COUNT($B$6:B68),"")</f>
         <v/>
       </c>
@@ -2890,7 +2920,7 @@
       <c r="O68" s="12"/>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A69" s="16" t="str">
+      <c r="A69" s="11" t="str">
         <f>IF(B69&lt;&gt;"",COUNT($B$6:B69),"")</f>
         <v/>
       </c>
@@ -2916,7 +2946,7 @@
       <c r="O69" s="12"/>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A70" s="16" t="str">
+      <c r="A70" s="11" t="str">
         <f>IF(B70&lt;&gt;"",COUNT($B$6:B70),"")</f>
         <v/>
       </c>
@@ -2942,7 +2972,7 @@
       <c r="O70" s="12"/>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A71" s="16" t="str">
+      <c r="A71" s="11" t="str">
         <f>IF(B71&lt;&gt;"",COUNT($B$6:B71),"")</f>
         <v/>
       </c>
@@ -2968,7 +2998,7 @@
       <c r="O71" s="12"/>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A72" s="16" t="str">
+      <c r="A72" s="11" t="str">
         <f>IF(B72&lt;&gt;"",COUNT($B$6:B72),"")</f>
         <v/>
       </c>
@@ -2994,7 +3024,7 @@
       <c r="O72" s="12"/>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A73" s="16" t="str">
+      <c r="A73" s="11" t="str">
         <f>IF(B73&lt;&gt;"",COUNT($B$6:B73),"")</f>
         <v/>
       </c>
@@ -3020,7 +3050,7 @@
       <c r="O73" s="12"/>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A74" s="16" t="str">
+      <c r="A74" s="11" t="str">
         <f>IF(B74&lt;&gt;"",COUNT($B$6:B74),"")</f>
         <v/>
       </c>
@@ -3046,7 +3076,7 @@
       <c r="O74" s="12"/>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A75" s="16" t="str">
+      <c r="A75" s="11" t="str">
         <f>IF(B75&lt;&gt;"",COUNT($B$6:B75),"")</f>
         <v/>
       </c>
@@ -3072,7 +3102,7 @@
       <c r="O75" s="12"/>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A76" s="16" t="str">
+      <c r="A76" s="11" t="str">
         <f>IF(B76&lt;&gt;"",COUNT($B$6:B76),"")</f>
         <v/>
       </c>
@@ -3098,7 +3128,7 @@
       <c r="O76" s="12"/>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A77" s="16" t="str">
+      <c r="A77" s="11" t="str">
         <f>IF(B77&lt;&gt;"",COUNT($B$6:B77),"")</f>
         <v/>
       </c>
@@ -3124,7 +3154,7 @@
       <c r="O77" s="12"/>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A78" s="16" t="str">
+      <c r="A78" s="11" t="str">
         <f>IF(B78&lt;&gt;"",COUNT($B$6:B78),"")</f>
         <v/>
       </c>
@@ -3150,7 +3180,7 @@
       <c r="O78" s="12"/>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A79" s="16" t="str">
+      <c r="A79" s="11" t="str">
         <f>IF(B79&lt;&gt;"",COUNT($B$6:B79),"")</f>
         <v/>
       </c>
@@ -3176,7 +3206,7 @@
       <c r="O79" s="12"/>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A80" s="16" t="str">
+      <c r="A80" s="11" t="str">
         <f>IF(B80&lt;&gt;"",COUNT($B$6:B80),"")</f>
         <v/>
       </c>
@@ -3202,7 +3232,7 @@
       <c r="O80" s="12"/>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A81" s="16" t="str">
+      <c r="A81" s="11" t="str">
         <f>IF(B81&lt;&gt;"",COUNT($B$6:B81),"")</f>
         <v/>
       </c>
@@ -3228,7 +3258,7 @@
       <c r="O81" s="12"/>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A82" s="16" t="str">
+      <c r="A82" s="11" t="str">
         <f>IF(B82&lt;&gt;"",COUNT($B$6:B82),"")</f>
         <v/>
       </c>
@@ -3254,7 +3284,7 @@
       <c r="O82" s="12"/>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A83" s="16" t="str">
+      <c r="A83" s="11" t="str">
         <f>IF(B83&lt;&gt;"",COUNT($B$6:B83),"")</f>
         <v/>
       </c>
@@ -3280,7 +3310,7 @@
       <c r="O83" s="12"/>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A84" s="16" t="str">
+      <c r="A84" s="11" t="str">
         <f>IF(B84&lt;&gt;"",COUNT($B$6:B84),"")</f>
         <v/>
       </c>
@@ -3306,7 +3336,7 @@
       <c r="O84" s="12"/>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A85" s="16" t="str">
+      <c r="A85" s="11" t="str">
         <f>IF(B85&lt;&gt;"",COUNT($B$6:B85),"")</f>
         <v/>
       </c>
@@ -3332,7 +3362,7 @@
       <c r="O85" s="12"/>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A86" s="16" t="str">
+      <c r="A86" s="11" t="str">
         <f>IF(B86&lt;&gt;"",COUNT($B$6:B86),"")</f>
         <v/>
       </c>
@@ -3358,7 +3388,7 @@
       <c r="O86" s="12"/>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A87" s="16" t="str">
+      <c r="A87" s="11" t="str">
         <f>IF(B87&lt;&gt;"",COUNT($B$6:B87),"")</f>
         <v/>
       </c>
@@ -3384,7 +3414,7 @@
       <c r="O87" s="12"/>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A88" s="16" t="str">
+      <c r="A88" s="11" t="str">
         <f>IF(B88&lt;&gt;"",COUNT($B$6:B88),"")</f>
         <v/>
       </c>
@@ -3410,7 +3440,7 @@
       <c r="O88" s="12"/>
     </row>
     <row r="89" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A89" s="16" t="str">
+      <c r="A89" s="11" t="str">
         <f>IF(B89&lt;&gt;"",COUNT($B$6:B89),"")</f>
         <v/>
       </c>
@@ -3436,7 +3466,7 @@
       <c r="O89" s="12"/>
     </row>
     <row r="90" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A90" s="16" t="str">
+      <c r="A90" s="11" t="str">
         <f>IF(B90&lt;&gt;"",COUNT($B$6:B90),"")</f>
         <v/>
       </c>
@@ -3462,7 +3492,7 @@
       <c r="O90" s="12"/>
     </row>
     <row r="91" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A91" s="16" t="str">
+      <c r="A91" s="11" t="str">
         <f>IF(B91&lt;&gt;"",COUNT($B$6:B91),"")</f>
         <v/>
       </c>
@@ -3488,7 +3518,7 @@
       <c r="O91" s="12"/>
     </row>
     <row r="92" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A92" s="16" t="str">
+      <c r="A92" s="11" t="str">
         <f>IF(B92&lt;&gt;"",COUNT($B$6:B92),"")</f>
         <v/>
       </c>
@@ -3514,7 +3544,7 @@
       <c r="O92" s="12"/>
     </row>
     <row r="93" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A93" s="16" t="str">
+      <c r="A93" s="11" t="str">
         <f>IF(B93&lt;&gt;"",COUNT($B$6:B93),"")</f>
         <v/>
       </c>
@@ -3540,7 +3570,7 @@
       <c r="O93" s="12"/>
     </row>
     <row r="94" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A94" s="16" t="str">
+      <c r="A94" s="11" t="str">
         <f>IF(B94&lt;&gt;"",COUNT($B$6:B94),"")</f>
         <v/>
       </c>
@@ -3566,7 +3596,7 @@
       <c r="O94" s="12"/>
     </row>
     <row r="95" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A95" s="16" t="str">
+      <c r="A95" s="11" t="str">
         <f>IF(B95&lt;&gt;"",COUNT($B$6:B95),"")</f>
         <v/>
       </c>
@@ -3592,7 +3622,7 @@
       <c r="O95" s="12"/>
     </row>
     <row r="96" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A96" s="16" t="str">
+      <c r="A96" s="11" t="str">
         <f>IF(B96&lt;&gt;"",COUNT($B$6:B96),"")</f>
         <v/>
       </c>
@@ -3618,7 +3648,7 @@
       <c r="O96" s="12"/>
     </row>
     <row r="97" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A97" s="16" t="str">
+      <c r="A97" s="11" t="str">
         <f>IF(B97&lt;&gt;"",COUNT($B$6:B97),"")</f>
         <v/>
       </c>
@@ -3644,7 +3674,7 @@
       <c r="O97" s="12"/>
     </row>
     <row r="98" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A98" s="16" t="str">
+      <c r="A98" s="11" t="str">
         <f>IF(B98&lt;&gt;"",COUNT($B$6:B98),"")</f>
         <v/>
       </c>
@@ -3670,7 +3700,7 @@
       <c r="O98" s="12"/>
     </row>
     <row r="99" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A99" s="16" t="str">
+      <c r="A99" s="11" t="str">
         <f>IF(B99&lt;&gt;"",COUNT($B$6:B99),"")</f>
         <v/>
       </c>
@@ -3696,7 +3726,7 @@
       <c r="O99" s="12"/>
     </row>
     <row r="100" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A100" s="16" t="str">
+      <c r="A100" s="11" t="str">
         <f>IF(B100&lt;&gt;"",COUNT($B$6:B100),"")</f>
         <v/>
       </c>
@@ -3722,7 +3752,7 @@
       <c r="O100" s="12"/>
     </row>
     <row r="101" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A101" s="16" t="str">
+      <c r="A101" s="11" t="str">
         <f>IF(B101&lt;&gt;"",COUNT($B$6:B101),"")</f>
         <v/>
       </c>
@@ -3748,7 +3778,7 @@
       <c r="O101" s="12"/>
     </row>
     <row r="102" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A102" s="16" t="str">
+      <c r="A102" s="11" t="str">
         <f>IF(B102&lt;&gt;"",COUNT($B$6:B102),"")</f>
         <v/>
       </c>
@@ -3774,7 +3804,7 @@
       <c r="O102" s="12"/>
     </row>
     <row r="103" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A103" s="16" t="str">
+      <c r="A103" s="11" t="str">
         <f>IF(B103&lt;&gt;"",COUNT($B$6:B103),"")</f>
         <v/>
       </c>
@@ -3800,7 +3830,7 @@
       <c r="O103" s="12"/>
     </row>
     <row r="104" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A104" s="16" t="str">
+      <c r="A104" s="11" t="str">
         <f>IF(B104&lt;&gt;"",COUNT($B$6:B104),"")</f>
         <v/>
       </c>
@@ -3826,7 +3856,7 @@
       <c r="O104" s="12"/>
     </row>
     <row r="105" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A105" s="16" t="str">
+      <c r="A105" s="11" t="str">
         <f>IF(B105&lt;&gt;"",COUNT($B$6:B105),"")</f>
         <v/>
       </c>
@@ -3852,7 +3882,7 @@
       <c r="O105" s="12"/>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A106" s="16" t="str">
+      <c r="A106" s="11" t="str">
         <f>IF(B106&lt;&gt;"",COUNT($B$6:B106),"")</f>
         <v/>
       </c>
@@ -3878,7 +3908,7 @@
       <c r="O106" s="12"/>
     </row>
     <row r="107" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A107" s="16" t="str">
+      <c r="A107" s="11" t="str">
         <f>IF(B107&lt;&gt;"",COUNT($B$6:B107),"")</f>
         <v/>
       </c>
@@ -3904,7 +3934,7 @@
       <c r="O107" s="12"/>
     </row>
     <row r="108" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A108" s="16" t="str">
+      <c r="A108" s="11" t="str">
         <f>IF(B108&lt;&gt;"",COUNT($B$6:B108),"")</f>
         <v/>
       </c>
@@ -3930,7 +3960,7 @@
       <c r="O108" s="12"/>
     </row>
     <row r="109" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A109" s="16" t="str">
+      <c r="A109" s="11" t="str">
         <f>IF(B109&lt;&gt;"",COUNT($B$6:B109),"")</f>
         <v/>
       </c>
@@ -3956,7 +3986,7 @@
       <c r="O109" s="12"/>
     </row>
     <row r="110" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A110" s="16" t="str">
+      <c r="A110" s="11" t="str">
         <f>IF(B110&lt;&gt;"",COUNT($B$6:B110),"")</f>
         <v/>
       </c>
@@ -3982,7 +4012,7 @@
       <c r="O110" s="12"/>
     </row>
     <row r="111" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A111" s="16" t="str">
+      <c r="A111" s="11" t="str">
         <f>IF(B111&lt;&gt;"",COUNT($B$6:B111),"")</f>
         <v/>
       </c>
@@ -4008,7 +4038,7 @@
       <c r="O111" s="12"/>
     </row>
     <row r="112" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A112" s="16" t="str">
+      <c r="A112" s="11" t="str">
         <f>IF(B112&lt;&gt;"",COUNT($B$6:B112),"")</f>
         <v/>
       </c>
@@ -4034,7 +4064,7 @@
       <c r="O112" s="12"/>
     </row>
     <row r="113" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A113" s="16" t="str">
+      <c r="A113" s="11" t="str">
         <f>IF(B113&lt;&gt;"",COUNT($B$6:B113),"")</f>
         <v/>
       </c>
@@ -4060,7 +4090,7 @@
       <c r="O113" s="12"/>
     </row>
     <row r="114" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A114" s="16" t="str">
+      <c r="A114" s="11" t="str">
         <f>IF(B114&lt;&gt;"",COUNT($B$6:B114),"")</f>
         <v/>
       </c>
@@ -4086,7 +4116,7 @@
       <c r="O114" s="12"/>
     </row>
     <row r="115" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A115" s="16" t="str">
+      <c r="A115" s="11" t="str">
         <f>IF(B115&lt;&gt;"",COUNT($B$6:B115),"")</f>
         <v/>
       </c>
@@ -4112,7 +4142,7 @@
       <c r="O115" s="12"/>
     </row>
     <row r="116" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A116" s="16" t="str">
+      <c r="A116" s="11" t="str">
         <f>IF(B116&lt;&gt;"",COUNT($B$6:B116),"")</f>
         <v/>
       </c>
@@ -4138,7 +4168,7 @@
       <c r="O116" s="12"/>
     </row>
     <row r="117" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A117" s="16" t="str">
+      <c r="A117" s="11" t="str">
         <f>IF(B117&lt;&gt;"",COUNT($B$6:B117),"")</f>
         <v/>
       </c>
@@ -4164,7 +4194,7 @@
       <c r="O117" s="12"/>
     </row>
     <row r="118" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A118" s="16" t="str">
+      <c r="A118" s="11" t="str">
         <f>IF(B118&lt;&gt;"",COUNT($B$6:B118),"")</f>
         <v/>
       </c>
@@ -4190,7 +4220,7 @@
       <c r="O118" s="12"/>
     </row>
     <row r="119" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A119" s="16" t="str">
+      <c r="A119" s="11" t="str">
         <f>IF(B119&lt;&gt;"",COUNT($B$6:B119),"")</f>
         <v/>
       </c>
@@ -4216,7 +4246,7 @@
       <c r="O119" s="12"/>
     </row>
     <row r="120" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A120" s="16" t="str">
+      <c r="A120" s="11" t="str">
         <f>IF(B120&lt;&gt;"",COUNT($B$6:B120),"")</f>
         <v/>
       </c>
@@ -4242,7 +4272,7 @@
       <c r="O120" s="12"/>
     </row>
     <row r="121" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A121" s="16" t="str">
+      <c r="A121" s="11" t="str">
         <f>IF(B121&lt;&gt;"",COUNT($B$6:B121),"")</f>
         <v/>
       </c>
@@ -4268,7 +4298,7 @@
       <c r="O121" s="12"/>
     </row>
     <row r="122" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A122" s="16" t="str">
+      <c r="A122" s="11" t="str">
         <f>IF(B122&lt;&gt;"",COUNT($B$6:B122),"")</f>
         <v/>
       </c>
@@ -4294,7 +4324,7 @@
       <c r="O122" s="12"/>
     </row>
     <row r="123" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A123" s="16" t="str">
+      <c r="A123" s="11" t="str">
         <f>IF(B123&lt;&gt;"",COUNT($B$6:B123),"")</f>
         <v/>
       </c>
@@ -4320,7 +4350,7 @@
       <c r="O123" s="12"/>
     </row>
     <row r="124" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A124" s="16" t="str">
+      <c r="A124" s="11" t="str">
         <f>IF(B124&lt;&gt;"",COUNT($B$6:B124),"")</f>
         <v/>
       </c>
@@ -4346,7 +4376,7 @@
       <c r="O124" s="12"/>
     </row>
     <row r="125" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A125" s="16" t="str">
+      <c r="A125" s="11" t="str">
         <f>IF(B125&lt;&gt;"",COUNT($B$6:B125),"")</f>
         <v/>
       </c>
@@ -4372,7 +4402,7 @@
       <c r="O125" s="12"/>
     </row>
     <row r="126" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A126" s="16" t="str">
+      <c r="A126" s="11" t="str">
         <f>IF(B126&lt;&gt;"",COUNT($B$6:B126),"")</f>
         <v/>
       </c>
@@ -4398,7 +4428,7 @@
       <c r="O126" s="12"/>
     </row>
     <row r="127" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A127" s="16" t="str">
+      <c r="A127" s="11" t="str">
         <f>IF(B127&lt;&gt;"",COUNT($B$6:B127),"")</f>
         <v/>
       </c>
@@ -4424,7 +4454,7 @@
       <c r="O127" s="12"/>
     </row>
     <row r="128" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A128" s="16" t="str">
+      <c r="A128" s="11" t="str">
         <f>IF(B128&lt;&gt;"",COUNT($B$6:B128),"")</f>
         <v/>
       </c>
@@ -4450,7 +4480,7 @@
       <c r="O128" s="12"/>
     </row>
     <row r="129" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A129" s="16" t="str">
+      <c r="A129" s="11" t="str">
         <f>IF(B129&lt;&gt;"",COUNT($B$6:B129),"")</f>
         <v/>
       </c>
@@ -4476,7 +4506,7 @@
       <c r="O129" s="12"/>
     </row>
     <row r="130" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A130" s="16" t="str">
+      <c r="A130" s="11" t="str">
         <f>IF(B130&lt;&gt;"",COUNT($B$6:B130),"")</f>
         <v/>
       </c>
@@ -4502,7 +4532,7 @@
       <c r="O130" s="12"/>
     </row>
     <row r="131" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A131" s="16" t="str">
+      <c r="A131" s="11" t="str">
         <f>IF(B131&lt;&gt;"",COUNT($B$6:B131),"")</f>
         <v/>
       </c>
@@ -4528,7 +4558,7 @@
       <c r="O131" s="12"/>
     </row>
     <row r="132" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A132" s="16" t="str">
+      <c r="A132" s="11" t="str">
         <f>IF(B132&lt;&gt;"",COUNT($B$6:B132),"")</f>
         <v/>
       </c>
@@ -4554,7 +4584,7 @@
       <c r="O132" s="12"/>
     </row>
     <row r="133" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A133" s="16" t="str">
+      <c r="A133" s="11" t="str">
         <f>IF(B133&lt;&gt;"",COUNT($B$6:B133),"")</f>
         <v/>
       </c>
@@ -4580,7 +4610,7 @@
       <c r="O133" s="12"/>
     </row>
     <row r="134" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A134" s="16" t="str">
+      <c r="A134" s="11" t="str">
         <f>IF(B134&lt;&gt;"",COUNT($B$6:B134),"")</f>
         <v/>
       </c>
@@ -4606,7 +4636,7 @@
       <c r="O134" s="12"/>
     </row>
     <row r="135" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A135" s="16" t="str">
+      <c r="A135" s="11" t="str">
         <f>IF(B135&lt;&gt;"",COUNT($B$6:B135),"")</f>
         <v/>
       </c>
@@ -4632,7 +4662,7 @@
       <c r="O135" s="12"/>
     </row>
     <row r="136" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A136" s="16" t="str">
+      <c r="A136" s="11" t="str">
         <f>IF(B136&lt;&gt;"",COUNT($B$6:B136),"")</f>
         <v/>
       </c>
@@ -4658,7 +4688,7 @@
       <c r="O136" s="12"/>
     </row>
     <row r="137" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A137" s="16" t="str">
+      <c r="A137" s="11" t="str">
         <f>IF(B137&lt;&gt;"",COUNT($B$6:B137),"")</f>
         <v/>
       </c>
@@ -4684,7 +4714,7 @@
       <c r="O137" s="12"/>
     </row>
     <row r="138" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A138" s="16" t="str">
+      <c r="A138" s="11" t="str">
         <f>IF(B138&lt;&gt;"",COUNT($B$6:B138),"")</f>
         <v/>
       </c>
@@ -4710,7 +4740,7 @@
       <c r="O138" s="12"/>
     </row>
     <row r="139" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A139" s="16" t="str">
+      <c r="A139" s="11" t="str">
         <f>IF(B139&lt;&gt;"",COUNT($B$6:B139),"")</f>
         <v/>
       </c>
@@ -4736,7 +4766,7 @@
       <c r="O139" s="12"/>
     </row>
     <row r="140" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A140" s="16" t="str">
+      <c r="A140" s="11" t="str">
         <f>IF(B140&lt;&gt;"",COUNT($B$6:B140),"")</f>
         <v/>
       </c>
@@ -4762,7 +4792,7 @@
       <c r="O140" s="12"/>
     </row>
     <row r="141" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A141" s="16" t="str">
+      <c r="A141" s="11" t="str">
         <f>IF(B141&lt;&gt;"",COUNT($B$6:B141),"")</f>
         <v/>
       </c>
@@ -4788,7 +4818,7 @@
       <c r="O141" s="12"/>
     </row>
     <row r="142" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A142" s="16" t="str">
+      <c r="A142" s="11" t="str">
         <f>IF(B142&lt;&gt;"",COUNT($B$6:B142),"")</f>
         <v/>
       </c>
@@ -4814,7 +4844,7 @@
       <c r="O142" s="12"/>
     </row>
     <row r="143" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A143" s="16" t="str">
+      <c r="A143" s="11" t="str">
         <f>IF(B143&lt;&gt;"",COUNT($B$6:B143),"")</f>
         <v/>
       </c>
@@ -4840,7 +4870,7 @@
       <c r="O143" s="12"/>
     </row>
     <row r="144" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A144" s="16" t="str">
+      <c r="A144" s="11" t="str">
         <f>IF(B144&lt;&gt;"",COUNT($B$6:B144),"")</f>
         <v/>
       </c>
@@ -4866,7 +4896,7 @@
       <c r="O144" s="12"/>
     </row>
     <row r="145" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A145" s="16" t="str">
+      <c r="A145" s="11" t="str">
         <f>IF(B145&lt;&gt;"",COUNT($B$6:B145),"")</f>
         <v/>
       </c>
@@ -4892,7 +4922,7 @@
       <c r="O145" s="12"/>
     </row>
     <row r="146" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A146" s="16" t="str">
+      <c r="A146" s="11" t="str">
         <f>IF(B146&lt;&gt;"",COUNT($B$6:B146),"")</f>
         <v/>
       </c>
@@ -4918,7 +4948,7 @@
       <c r="O146" s="12"/>
     </row>
     <row r="147" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A147" s="16" t="str">
+      <c r="A147" s="11" t="str">
         <f>IF(B147&lt;&gt;"",COUNT($B$6:B147),"")</f>
         <v/>
       </c>
@@ -4944,7 +4974,7 @@
       <c r="O147" s="12"/>
     </row>
     <row r="148" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A148" s="16" t="str">
+      <c r="A148" s="11" t="str">
         <f>IF(B148&lt;&gt;"",COUNT($B$6:B148),"")</f>
         <v/>
       </c>
@@ -4970,7 +5000,7 @@
       <c r="O148" s="12"/>
     </row>
     <row r="149" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A149" s="16" t="str">
+      <c r="A149" s="11" t="str">
         <f>IF(B149&lt;&gt;"",COUNT($B$6:B149),"")</f>
         <v/>
       </c>
@@ -4996,7 +5026,7 @@
       <c r="O149" s="12"/>
     </row>
     <row r="150" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A150" s="16" t="str">
+      <c r="A150" s="11" t="str">
         <f>IF(B150&lt;&gt;"",COUNT($B$6:B150),"")</f>
         <v/>
       </c>
@@ -5022,7 +5052,7 @@
       <c r="O150" s="12"/>
     </row>
     <row r="151" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A151" s="16" t="str">
+      <c r="A151" s="11" t="str">
         <f>IF(B151&lt;&gt;"",COUNT($B$6:B151),"")</f>
         <v/>
       </c>
@@ -5048,7 +5078,7 @@
       <c r="O151" s="12"/>
     </row>
     <row r="152" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A152" s="16" t="str">
+      <c r="A152" s="11" t="str">
         <f>IF(B152&lt;&gt;"",COUNT($B$6:B152),"")</f>
         <v/>
       </c>
@@ -5074,7 +5104,7 @@
       <c r="O152" s="12"/>
     </row>
     <row r="153" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A153" s="16" t="str">
+      <c r="A153" s="11" t="str">
         <f>IF(B153&lt;&gt;"",COUNT($B$6:B153),"")</f>
         <v/>
       </c>
@@ -5100,7 +5130,7 @@
       <c r="O153" s="12"/>
     </row>
     <row r="154" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A154" s="16" t="str">
+      <c r="A154" s="11" t="str">
         <f>IF(B154&lt;&gt;"",COUNT($B$6:B154),"")</f>
         <v/>
       </c>
@@ -5126,7 +5156,7 @@
       <c r="O154" s="12"/>
     </row>
     <row r="155" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A155" s="16" t="str">
+      <c r="A155" s="11" t="str">
         <f>IF(B155&lt;&gt;"",COUNT($B$6:B155),"")</f>
         <v/>
       </c>
@@ -5152,7 +5182,7 @@
       <c r="O155" s="12"/>
     </row>
     <row r="156" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A156" s="16" t="str">
+      <c r="A156" s="11" t="str">
         <f>IF(B156&lt;&gt;"",COUNT($B$6:B156),"")</f>
         <v/>
       </c>
@@ -5178,7 +5208,7 @@
       <c r="O156" s="12"/>
     </row>
     <row r="157" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A157" s="16" t="str">
+      <c r="A157" s="11" t="str">
         <f>IF(B157&lt;&gt;"",COUNT($B$6:B157),"")</f>
         <v/>
       </c>
@@ -5204,7 +5234,7 @@
       <c r="O157" s="12"/>
     </row>
     <row r="158" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A158" s="16" t="str">
+      <c r="A158" s="11" t="str">
         <f>IF(B158&lt;&gt;"",COUNT($B$6:B158),"")</f>
         <v/>
       </c>
@@ -5230,7 +5260,7 @@
       <c r="O158" s="12"/>
     </row>
     <row r="159" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A159" s="16" t="str">
+      <c r="A159" s="11" t="str">
         <f>IF(B159&lt;&gt;"",COUNT($B$6:B159),"")</f>
         <v/>
       </c>
@@ -5256,7 +5286,7 @@
       <c r="O159" s="12"/>
     </row>
     <row r="160" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A160" s="16" t="str">
+      <c r="A160" s="11" t="str">
         <f>IF(B160&lt;&gt;"",COUNT($B$6:B160),"")</f>
         <v/>
       </c>
@@ -5282,7 +5312,7 @@
       <c r="O160" s="12"/>
     </row>
     <row r="161" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A161" s="16" t="str">
+      <c r="A161" s="11" t="str">
         <f>IF(B161&lt;&gt;"",COUNT($B$6:B161),"")</f>
         <v/>
       </c>
@@ -5308,7 +5338,7 @@
       <c r="O161" s="12"/>
     </row>
     <row r="162" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A162" s="16" t="str">
+      <c r="A162" s="11" t="str">
         <f>IF(B162&lt;&gt;"",COUNT($B$6:B162),"")</f>
         <v/>
       </c>
@@ -5334,7 +5364,7 @@
       <c r="O162" s="12"/>
     </row>
     <row r="163" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A163" s="16" t="str">
+      <c r="A163" s="11" t="str">
         <f>IF(B163&lt;&gt;"",COUNT($B$6:B163),"")</f>
         <v/>
       </c>
@@ -5360,7 +5390,7 @@
       <c r="O163" s="12"/>
     </row>
     <row r="164" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A164" s="16" t="str">
+      <c r="A164" s="11" t="str">
         <f>IF(B164&lt;&gt;"",COUNT($B$6:B164),"")</f>
         <v/>
       </c>
@@ -5386,7 +5416,7 @@
       <c r="O164" s="12"/>
     </row>
     <row r="165" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A165" s="16" t="str">
+      <c r="A165" s="11" t="str">
         <f>IF(B165&lt;&gt;"",COUNT($B$6:B165),"")</f>
         <v/>
       </c>
@@ -5412,7 +5442,7 @@
       <c r="O165" s="12"/>
     </row>
     <row r="166" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A166" s="16" t="str">
+      <c r="A166" s="11" t="str">
         <f>IF(B166&lt;&gt;"",COUNT($B$6:B166),"")</f>
         <v/>
       </c>
@@ -5438,7 +5468,7 @@
       <c r="O166" s="12"/>
     </row>
     <row r="167" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A167" s="16" t="str">
+      <c r="A167" s="11" t="str">
         <f>IF(B167&lt;&gt;"",COUNT($B$6:B167),"")</f>
         <v/>
       </c>
@@ -5464,7 +5494,7 @@
       <c r="O167" s="12"/>
     </row>
     <row r="168" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A168" s="16" t="str">
+      <c r="A168" s="11" t="str">
         <f>IF(B168&lt;&gt;"",COUNT($B$6:B168),"")</f>
         <v/>
       </c>
@@ -5490,7 +5520,7 @@
       <c r="O168" s="12"/>
     </row>
     <row r="169" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A169" s="16" t="str">
+      <c r="A169" s="11" t="str">
         <f>IF(B169&lt;&gt;"",COUNT($B$6:B169),"")</f>
         <v/>
       </c>
@@ -5516,7 +5546,7 @@
       <c r="O169" s="12"/>
     </row>
     <row r="170" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A170" s="16" t="str">
+      <c r="A170" s="11" t="str">
         <f>IF(B170&lt;&gt;"",COUNT($B$6:B170),"")</f>
         <v/>
       </c>
@@ -5542,7 +5572,7 @@
       <c r="O170" s="12"/>
     </row>
     <row r="171" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A171" s="16" t="str">
+      <c r="A171" s="11" t="str">
         <f>IF(B171&lt;&gt;"",COUNT($B$6:B171),"")</f>
         <v/>
       </c>
@@ -5568,7 +5598,7 @@
       <c r="O171" s="12"/>
     </row>
     <row r="172" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A172" s="16" t="str">
+      <c r="A172" s="11" t="str">
         <f>IF(B172&lt;&gt;"",COUNT($B$6:B172),"")</f>
         <v/>
       </c>
@@ -5594,7 +5624,7 @@
       <c r="O172" s="12"/>
     </row>
     <row r="173" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A173" s="16" t="str">
+      <c r="A173" s="11" t="str">
         <f>IF(B173&lt;&gt;"",COUNT($B$6:B173),"")</f>
         <v/>
       </c>
@@ -5620,7 +5650,7 @@
       <c r="O173" s="12"/>
     </row>
     <row r="174" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A174" s="16" t="str">
+      <c r="A174" s="11" t="str">
         <f>IF(B174&lt;&gt;"",COUNT($B$6:B174),"")</f>
         <v/>
       </c>
@@ -5646,7 +5676,7 @@
       <c r="O174" s="12"/>
     </row>
     <row r="175" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A175" s="16" t="str">
+      <c r="A175" s="11" t="str">
         <f>IF(B175&lt;&gt;"",COUNT($B$6:B175),"")</f>
         <v/>
       </c>
@@ -5672,7 +5702,7 @@
       <c r="O175" s="12"/>
     </row>
     <row r="176" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A176" s="16" t="str">
+      <c r="A176" s="11" t="str">
         <f>IF(B176&lt;&gt;"",COUNT($B$6:B176),"")</f>
         <v/>
       </c>
@@ -5698,7 +5728,7 @@
       <c r="O176" s="12"/>
     </row>
     <row r="177" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A177" s="16" t="str">
+      <c r="A177" s="11" t="str">
         <f>IF(B177&lt;&gt;"",COUNT($B$6:B177),"")</f>
         <v/>
       </c>
@@ -5724,7 +5754,7 @@
       <c r="O177" s="12"/>
     </row>
     <row r="178" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A178" s="16" t="str">
+      <c r="A178" s="11" t="str">
         <f>IF(B178&lt;&gt;"",COUNT($B$6:B178),"")</f>
         <v/>
       </c>
@@ -5750,7 +5780,7 @@
       <c r="O178" s="12"/>
     </row>
     <row r="179" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A179" s="16" t="str">
+      <c r="A179" s="11" t="str">
         <f>IF(B179&lt;&gt;"",COUNT($B$6:B179),"")</f>
         <v/>
       </c>
@@ -5776,7 +5806,7 @@
       <c r="O179" s="12"/>
     </row>
     <row r="180" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A180" s="16" t="str">
+      <c r="A180" s="11" t="str">
         <f>IF(B180&lt;&gt;"",COUNT($B$6:B180),"")</f>
         <v/>
       </c>
@@ -5802,7 +5832,7 @@
       <c r="O180" s="12"/>
     </row>
     <row r="181" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A181" s="16" t="str">
+      <c r="A181" s="11" t="str">
         <f>IF(B181&lt;&gt;"",COUNT($B$6:B181),"")</f>
         <v/>
       </c>
@@ -5828,7 +5858,7 @@
       <c r="O181" s="12"/>
     </row>
     <row r="182" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A182" s="16" t="str">
+      <c r="A182" s="11" t="str">
         <f>IF(B182&lt;&gt;"",COUNT($B$6:B182),"")</f>
         <v/>
       </c>
@@ -5854,7 +5884,7 @@
       <c r="O182" s="12"/>
     </row>
     <row r="183" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A183" s="16" t="str">
+      <c r="A183" s="11" t="str">
         <f>IF(B183&lt;&gt;"",COUNT($B$6:B183),"")</f>
         <v/>
       </c>
@@ -5880,7 +5910,7 @@
       <c r="O183" s="12"/>
     </row>
     <row r="184" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A184" s="16" t="str">
+      <c r="A184" s="11" t="str">
         <f>IF(B184&lt;&gt;"",COUNT($B$6:B184),"")</f>
         <v/>
       </c>
@@ -5906,7 +5936,7 @@
       <c r="O184" s="12"/>
     </row>
     <row r="185" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A185" s="16" t="str">
+      <c r="A185" s="11" t="str">
         <f>IF(B185&lt;&gt;"",COUNT($B$6:B185),"")</f>
         <v/>
       </c>
@@ -5932,7 +5962,7 @@
       <c r="O185" s="12"/>
     </row>
     <row r="186" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A186" s="16" t="str">
+      <c r="A186" s="11" t="str">
         <f>IF(B186&lt;&gt;"",COUNT($B$6:B186),"")</f>
         <v/>
       </c>
@@ -5958,7 +5988,7 @@
       <c r="O186" s="12"/>
     </row>
     <row r="187" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A187" s="16" t="str">
+      <c r="A187" s="11" t="str">
         <f>IF(B187&lt;&gt;"",COUNT($B$6:B187),"")</f>
         <v/>
       </c>
@@ -5984,7 +6014,7 @@
       <c r="O187" s="12"/>
     </row>
     <row r="188" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A188" s="16" t="str">
+      <c r="A188" s="11" t="str">
         <f>IF(B188&lt;&gt;"",COUNT($B$6:B188),"")</f>
         <v/>
       </c>
@@ -6010,7 +6040,7 @@
       <c r="O188" s="12"/>
     </row>
     <row r="189" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A189" s="16" t="str">
+      <c r="A189" s="11" t="str">
         <f>IF(B189&lt;&gt;"",COUNT($B$6:B189),"")</f>
         <v/>
       </c>
@@ -6036,7 +6066,7 @@
       <c r="O189" s="12"/>
     </row>
     <row r="190" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A190" s="16" t="str">
+      <c r="A190" s="11" t="str">
         <f>IF(B190&lt;&gt;"",COUNT($B$6:B190),"")</f>
         <v/>
       </c>
@@ -6062,7 +6092,7 @@
       <c r="O190" s="12"/>
     </row>
     <row r="191" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A191" s="16" t="str">
+      <c r="A191" s="11" t="str">
         <f>IF(B191&lt;&gt;"",COUNT($B$6:B191),"")</f>
         <v/>
       </c>
@@ -6088,7 +6118,7 @@
       <c r="O191" s="12"/>
     </row>
     <row r="192" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A192" s="16" t="str">
+      <c r="A192" s="11" t="str">
         <f>IF(B192&lt;&gt;"",COUNT($B$6:B192),"")</f>
         <v/>
       </c>
@@ -6114,7 +6144,7 @@
       <c r="O192" s="12"/>
     </row>
     <row r="193" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A193" s="16" t="str">
+      <c r="A193" s="11" t="str">
         <f>IF(B193&lt;&gt;"",COUNT($B$6:B193),"")</f>
         <v/>
       </c>
@@ -6140,7 +6170,7 @@
       <c r="O193" s="12"/>
     </row>
     <row r="194" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A194" s="16" t="str">
+      <c r="A194" s="11" t="str">
         <f>IF(B194&lt;&gt;"",COUNT($B$6:B194),"")</f>
         <v/>
       </c>
@@ -6166,7 +6196,7 @@
       <c r="O194" s="12"/>
     </row>
     <row r="195" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A195" s="16" t="str">
+      <c r="A195" s="11" t="str">
         <f>IF(B195&lt;&gt;"",COUNT($B$6:B195),"")</f>
         <v/>
       </c>
@@ -6192,7 +6222,7 @@
       <c r="O195" s="12"/>
     </row>
     <row r="196" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A196" s="16" t="str">
+      <c r="A196" s="11" t="str">
         <f>IF(B196&lt;&gt;"",COUNT($B$6:B196),"")</f>
         <v/>
       </c>
@@ -6218,7 +6248,7 @@
       <c r="O196" s="12"/>
     </row>
     <row r="197" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A197" s="16" t="str">
+      <c r="A197" s="11" t="str">
         <f>IF(B197&lt;&gt;"",COUNT($B$6:B197),"")</f>
         <v/>
       </c>
@@ -6244,7 +6274,7 @@
       <c r="O197" s="12"/>
     </row>
     <row r="198" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A198" s="16" t="str">
+      <c r="A198" s="11" t="str">
         <f>IF(B198&lt;&gt;"",COUNT($B$6:B198),"")</f>
         <v/>
       </c>
@@ -6270,7 +6300,7 @@
       <c r="O198" s="12"/>
     </row>
     <row r="199" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A199" s="16" t="str">
+      <c r="A199" s="11" t="str">
         <f>IF(B199&lt;&gt;"",COUNT($B$6:B199),"")</f>
         <v/>
       </c>
@@ -6296,7 +6326,7 @@
       <c r="O199" s="12"/>
     </row>
     <row r="200" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A200" s="16" t="str">
+      <c r="A200" s="11" t="str">
         <f>IF(B200&lt;&gt;"",COUNT($B$6:B200),"")</f>
         <v/>
       </c>
@@ -6322,7 +6352,7 @@
       <c r="O200" s="12"/>
     </row>
     <row r="201" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A201" s="16" t="str">
+      <c r="A201" s="11" t="str">
         <f>IF(B201&lt;&gt;"",COUNT($B$6:B201),"")</f>
         <v/>
       </c>
@@ -6348,7 +6378,7 @@
       <c r="O201" s="12"/>
     </row>
     <row r="202" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A202" s="16" t="str">
+      <c r="A202" s="11" t="str">
         <f>IF(B202&lt;&gt;"",COUNT($B$6:B202),"")</f>
         <v/>
       </c>
@@ -6374,7 +6404,7 @@
       <c r="O202" s="12"/>
     </row>
     <row r="203" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A203" s="16" t="str">
+      <c r="A203" s="11" t="str">
         <f>IF(B203&lt;&gt;"",COUNT($B$6:B203),"")</f>
         <v/>
       </c>
@@ -6400,7 +6430,7 @@
       <c r="O203" s="12"/>
     </row>
     <row r="204" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A204" s="16" t="str">
+      <c r="A204" s="11" t="str">
         <f>IF(B204&lt;&gt;"",COUNT($B$6:B204),"")</f>
         <v/>
       </c>
@@ -6426,7 +6456,7 @@
       <c r="O204" s="12"/>
     </row>
     <row r="205" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A205" s="16" t="str">
+      <c r="A205" s="11" t="str">
         <f>IF(B205&lt;&gt;"",COUNT($B$6:B205),"")</f>
         <v/>
       </c>
@@ -6452,7 +6482,7 @@
       <c r="O205" s="12"/>
     </row>
     <row r="206" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A206" s="16" t="str">
+      <c r="A206" s="11" t="str">
         <f>IF(B206&lt;&gt;"",COUNT($B$6:B206),"")</f>
         <v/>
       </c>
@@ -6478,7 +6508,7 @@
       <c r="O206" s="12"/>
     </row>
     <row r="207" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A207" s="16" t="str">
+      <c r="A207" s="11" t="str">
         <f>IF(B207&lt;&gt;"",COUNT($B$6:B207),"")</f>
         <v/>
       </c>
@@ -6504,7 +6534,7 @@
       <c r="O207" s="12"/>
     </row>
     <row r="208" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A208" s="16" t="str">
+      <c r="A208" s="11" t="str">
         <f>IF(B208&lt;&gt;"",COUNT($B$6:B208),"")</f>
         <v/>
       </c>
@@ -6530,7 +6560,7 @@
       <c r="O208" s="12"/>
     </row>
     <row r="209" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A209" s="16" t="str">
+      <c r="A209" s="11" t="str">
         <f>IF(B209&lt;&gt;"",COUNT($B$6:B209),"")</f>
         <v/>
       </c>
@@ -6556,7 +6586,7 @@
       <c r="O209" s="12"/>
     </row>
     <row r="210" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A210" s="16" t="str">
+      <c r="A210" s="11" t="str">
         <f>IF(B210&lt;&gt;"",COUNT($B$6:B210),"")</f>
         <v/>
       </c>
@@ -6582,7 +6612,7 @@
       <c r="O210" s="12"/>
     </row>
     <row r="211" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A211" s="16" t="str">
+      <c r="A211" s="11" t="str">
         <f>IF(B211&lt;&gt;"",COUNT($B$6:B211),"")</f>
         <v/>
       </c>
@@ -6608,7 +6638,7 @@
       <c r="O211" s="12"/>
     </row>
     <row r="212" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A212" s="16" t="str">
+      <c r="A212" s="11" t="str">
         <f>IF(B212&lt;&gt;"",COUNT($B$6:B212),"")</f>
         <v/>
       </c>
@@ -6634,7 +6664,7 @@
       <c r="O212" s="12"/>
     </row>
     <row r="213" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A213" s="16" t="str">
+      <c r="A213" s="11" t="str">
         <f>IF(B213&lt;&gt;"",COUNT($B$6:B213),"")</f>
         <v/>
       </c>
@@ -6660,7 +6690,7 @@
       <c r="O213" s="12"/>
     </row>
     <row r="214" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A214" s="16" t="str">
+      <c r="A214" s="11" t="str">
         <f>IF(B214&lt;&gt;"",COUNT($B$6:B214),"")</f>
         <v/>
       </c>
@@ -6686,7 +6716,7 @@
       <c r="O214" s="12"/>
     </row>
     <row r="215" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A215" s="16" t="str">
+      <c r="A215" s="11" t="str">
         <f>IF(B215&lt;&gt;"",COUNT($B$6:B215),"")</f>
         <v/>
       </c>
@@ -6712,7 +6742,7 @@
       <c r="O215" s="12"/>
     </row>
     <row r="216" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A216" s="16" t="str">
+      <c r="A216" s="11" t="str">
         <f>IF(B216&lt;&gt;"",COUNT($B$6:B216),"")</f>
         <v/>
       </c>
@@ -6738,7 +6768,7 @@
       <c r="O216" s="12"/>
     </row>
     <row r="217" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A217" s="16" t="str">
+      <c r="A217" s="11" t="str">
         <f>IF(B217&lt;&gt;"",COUNT($B$6:B217),"")</f>
         <v/>
       </c>
@@ -6764,7 +6794,7 @@
       <c r="O217" s="12"/>
     </row>
     <row r="218" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A218" s="16" t="str">
+      <c r="A218" s="11" t="str">
         <f>IF(B218&lt;&gt;"",COUNT($B$6:B218),"")</f>
         <v/>
       </c>
@@ -6790,7 +6820,7 @@
       <c r="O218" s="12"/>
     </row>
     <row r="219" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A219" s="16" t="str">
+      <c r="A219" s="11" t="str">
         <f>IF(B219&lt;&gt;"",COUNT($B$6:B219),"")</f>
         <v/>
       </c>
@@ -6816,7 +6846,7 @@
       <c r="O219" s="12"/>
     </row>
     <row r="220" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A220" s="16" t="str">
+      <c r="A220" s="11" t="str">
         <f>IF(B220&lt;&gt;"",COUNT($B$6:B220),"")</f>
         <v/>
       </c>
@@ -6842,7 +6872,7 @@
       <c r="O220" s="12"/>
     </row>
     <row r="221" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A221" s="16" t="str">
+      <c r="A221" s="11" t="str">
         <f>IF(B221&lt;&gt;"",COUNT($B$6:B221),"")</f>
         <v/>
       </c>
@@ -6868,7 +6898,7 @@
       <c r="O221" s="12"/>
     </row>
     <row r="222" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A222" s="16" t="str">
+      <c r="A222" s="11" t="str">
         <f>IF(B222&lt;&gt;"",COUNT($B$6:B222),"")</f>
         <v/>
       </c>
@@ -6894,7 +6924,7 @@
       <c r="O222" s="12"/>
     </row>
     <row r="223" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A223" s="16" t="str">
+      <c r="A223" s="11" t="str">
         <f>IF(B223&lt;&gt;"",COUNT($B$6:B223),"")</f>
         <v/>
       </c>
@@ -6920,7 +6950,7 @@
       <c r="O223" s="12"/>
     </row>
     <row r="224" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A224" s="16" t="str">
+      <c r="A224" s="11" t="str">
         <f>IF(B224&lt;&gt;"",COUNT($B$6:B224),"")</f>
         <v/>
       </c>
@@ -6946,7 +6976,7 @@
       <c r="O224" s="12"/>
     </row>
     <row r="225" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A225" s="16" t="str">
+      <c r="A225" s="11" t="str">
         <f>IF(B225&lt;&gt;"",COUNT($B$6:B225),"")</f>
         <v/>
       </c>
@@ -6972,7 +7002,7 @@
       <c r="O225" s="12"/>
     </row>
     <row r="226" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A226" s="16" t="str">
+      <c r="A226" s="11" t="str">
         <f>IF(B226&lt;&gt;"",COUNT($B$6:B226),"")</f>
         <v/>
       </c>
@@ -6998,7 +7028,7 @@
       <c r="O226" s="12"/>
     </row>
     <row r="227" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A227" s="16" t="str">
+      <c r="A227" s="11" t="str">
         <f>IF(B227&lt;&gt;"",COUNT($B$6:B227),"")</f>
         <v/>
       </c>
@@ -7024,7 +7054,7 @@
       <c r="O227" s="12"/>
     </row>
     <row r="228" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A228" s="16" t="str">
+      <c r="A228" s="11" t="str">
         <f>IF(B228&lt;&gt;"",COUNT($B$6:B228),"")</f>
         <v/>
       </c>
@@ -7050,7 +7080,7 @@
       <c r="O228" s="12"/>
     </row>
     <row r="229" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A229" s="16" t="str">
+      <c r="A229" s="11" t="str">
         <f>IF(B229&lt;&gt;"",COUNT($B$6:B229),"")</f>
         <v/>
       </c>
@@ -7076,7 +7106,7 @@
       <c r="O229" s="12"/>
     </row>
     <row r="230" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A230" s="16" t="str">
+      <c r="A230" s="11" t="str">
         <f>IF(B230&lt;&gt;"",COUNT($B$6:B230),"")</f>
         <v/>
       </c>
@@ -7102,7 +7132,7 @@
       <c r="O230" s="12"/>
     </row>
     <row r="231" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A231" s="16" t="str">
+      <c r="A231" s="11" t="str">
         <f>IF(B231&lt;&gt;"",COUNT($B$6:B231),"")</f>
         <v/>
       </c>
@@ -7128,7 +7158,7 @@
       <c r="O231" s="12"/>
     </row>
     <row r="232" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A232" s="16" t="str">
+      <c r="A232" s="11" t="str">
         <f>IF(B232&lt;&gt;"",COUNT($B$6:B232),"")</f>
         <v/>
       </c>
@@ -7154,7 +7184,7 @@
       <c r="O232" s="12"/>
     </row>
     <row r="233" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A233" s="16" t="str">
+      <c r="A233" s="11" t="str">
         <f>IF(B233&lt;&gt;"",COUNT($B$6:B233),"")</f>
         <v/>
       </c>
@@ -7180,7 +7210,7 @@
       <c r="O233" s="12"/>
     </row>
     <row r="234" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A234" s="16" t="str">
+      <c r="A234" s="11" t="str">
         <f>IF(B234&lt;&gt;"",COUNT($B$6:B234),"")</f>
         <v/>
       </c>
@@ -7206,7 +7236,7 @@
       <c r="O234" s="12"/>
     </row>
     <row r="235" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A235" s="16" t="str">
+      <c r="A235" s="11" t="str">
         <f>IF(B235&lt;&gt;"",COUNT($B$6:B235),"")</f>
         <v/>
       </c>
@@ -7232,7 +7262,7 @@
       <c r="O235" s="12"/>
     </row>
     <row r="236" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A236" s="16" t="str">
+      <c r="A236" s="11" t="str">
         <f>IF(B236&lt;&gt;"",COUNT($B$6:B236),"")</f>
         <v/>
       </c>
@@ -7258,7 +7288,7 @@
       <c r="O236" s="12"/>
     </row>
     <row r="237" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A237" s="16" t="str">
+      <c r="A237" s="11" t="str">
         <f>IF(B237&lt;&gt;"",COUNT($B$6:B237),"")</f>
         <v/>
       </c>
@@ -7284,7 +7314,7 @@
       <c r="O237" s="12"/>
     </row>
     <row r="238" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A238" s="16" t="str">
+      <c r="A238" s="11" t="str">
         <f>IF(B238&lt;&gt;"",COUNT($B$6:B238),"")</f>
         <v/>
       </c>
@@ -7310,7 +7340,7 @@
       <c r="O238" s="12"/>
     </row>
     <row r="239" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A239" s="16" t="str">
+      <c r="A239" s="11" t="str">
         <f>IF(B239&lt;&gt;"",COUNT($B$6:B239),"")</f>
         <v/>
       </c>
@@ -7336,7 +7366,7 @@
       <c r="O239" s="12"/>
     </row>
     <row r="240" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A240" s="16" t="str">
+      <c r="A240" s="11" t="str">
         <f>IF(B240&lt;&gt;"",COUNT($B$6:B240),"")</f>
         <v/>
       </c>
@@ -7362,7 +7392,7 @@
       <c r="O240" s="12"/>
     </row>
     <row r="241" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A241" s="16" t="str">
+      <c r="A241" s="11" t="str">
         <f>IF(B241&lt;&gt;"",COUNT($B$6:B241),"")</f>
         <v/>
       </c>
@@ -7388,7 +7418,7 @@
       <c r="O241" s="12"/>
     </row>
     <row r="242" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A242" s="16" t="str">
+      <c r="A242" s="11" t="str">
         <f>IF(B242&lt;&gt;"",COUNT($B$6:B242),"")</f>
         <v/>
       </c>
@@ -7414,7 +7444,7 @@
       <c r="O242" s="12"/>
     </row>
     <row r="243" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A243" s="16" t="str">
+      <c r="A243" s="11" t="str">
         <f>IF(B243&lt;&gt;"",COUNT($B$6:B243),"")</f>
         <v/>
       </c>
@@ -7440,7 +7470,7 @@
       <c r="O243" s="12"/>
     </row>
     <row r="244" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A244" s="16" t="str">
+      <c r="A244" s="11" t="str">
         <f>IF(B244&lt;&gt;"",COUNT($B$6:B244),"")</f>
         <v/>
       </c>
@@ -7466,7 +7496,7 @@
       <c r="O244" s="12"/>
     </row>
     <row r="245" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A245" s="16" t="str">
+      <c r="A245" s="11" t="str">
         <f>IF(B245&lt;&gt;"",COUNT($B$6:B245),"")</f>
         <v/>
       </c>
@@ -7492,7 +7522,7 @@
       <c r="O245" s="12"/>
     </row>
     <row r="246" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A246" s="16" t="str">
+      <c r="A246" s="11" t="str">
         <f>IF(B246&lt;&gt;"",COUNT($B$6:B246),"")</f>
         <v/>
       </c>
@@ -7518,7 +7548,7 @@
       <c r="O246" s="12"/>
     </row>
     <row r="247" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A247" s="16" t="str">
+      <c r="A247" s="11" t="str">
         <f>IF(B247&lt;&gt;"",COUNT($B$6:B247),"")</f>
         <v/>
       </c>
@@ -7544,7 +7574,7 @@
       <c r="O247" s="12"/>
     </row>
     <row r="248" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A248" s="16" t="str">
+      <c r="A248" s="11" t="str">
         <f>IF(B248&lt;&gt;"",COUNT($B$6:B248),"")</f>
         <v/>
       </c>
@@ -7570,7 +7600,7 @@
       <c r="O248" s="12"/>
     </row>
     <row r="249" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A249" s="16" t="str">
+      <c r="A249" s="11" t="str">
         <f>IF(B249&lt;&gt;"",COUNT($B$6:B249),"")</f>
         <v/>
       </c>
@@ -7596,7 +7626,7 @@
       <c r="O249" s="12"/>
     </row>
     <row r="250" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A250" s="16" t="str">
+      <c r="A250" s="11" t="str">
         <f>IF(B250&lt;&gt;"",COUNT($B$6:B250),"")</f>
         <v/>
       </c>
@@ -7622,7 +7652,7 @@
       <c r="O250" s="12"/>
     </row>
     <row r="251" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A251" s="16" t="str">
+      <c r="A251" s="11" t="str">
         <f>IF(B251&lt;&gt;"",COUNT($B$6:B251),"")</f>
         <v/>
       </c>
@@ -7648,7 +7678,7 @@
       <c r="O251" s="12"/>
     </row>
     <row r="252" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A252" s="16" t="str">
+      <c r="A252" s="11" t="str">
         <f>IF(B252&lt;&gt;"",COUNT($B$6:B252),"")</f>
         <v/>
       </c>
@@ -7674,7 +7704,7 @@
       <c r="O252" s="12"/>
     </row>
     <row r="253" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A253" s="16" t="str">
+      <c r="A253" s="11" t="str">
         <f>IF(B253&lt;&gt;"",COUNT($B$6:B253),"")</f>
         <v/>
       </c>
@@ -7700,7 +7730,7 @@
       <c r="O253" s="12"/>
     </row>
     <row r="254" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A254" s="16" t="str">
+      <c r="A254" s="11" t="str">
         <f>IF(B254&lt;&gt;"",COUNT($B$6:B254),"")</f>
         <v/>
       </c>
@@ -7726,7 +7756,7 @@
       <c r="O254" s="12"/>
     </row>
     <row r="255" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A255" s="16" t="str">
+      <c r="A255" s="11" t="str">
         <f>IF(B255&lt;&gt;"",COUNT($B$6:B255),"")</f>
         <v/>
       </c>
@@ -7752,7 +7782,7 @@
       <c r="O255" s="12"/>
     </row>
     <row r="256" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A256" s="16" t="str">
+      <c r="A256" s="11" t="str">
         <f>IF(B256&lt;&gt;"",COUNT($B$6:B256),"")</f>
         <v/>
       </c>
@@ -7778,7 +7808,7 @@
       <c r="O256" s="12"/>
     </row>
     <row r="257" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A257" s="16" t="str">
+      <c r="A257" s="11" t="str">
         <f>IF(B257&lt;&gt;"",COUNT($B$6:B257),"")</f>
         <v/>
       </c>
@@ -7804,7 +7834,7 @@
       <c r="O257" s="12"/>
     </row>
     <row r="258" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A258" s="16" t="str">
+      <c r="A258" s="11" t="str">
         <f>IF(B258&lt;&gt;"",COUNT($B$6:B258),"")</f>
         <v/>
       </c>
@@ -7830,7 +7860,7 @@
       <c r="O258" s="12"/>
     </row>
     <row r="259" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A259" s="16" t="str">
+      <c r="A259" s="11" t="str">
         <f>IF(B259&lt;&gt;"",COUNT($B$6:B259),"")</f>
         <v/>
       </c>
@@ -7856,7 +7886,7 @@
       <c r="O259" s="12"/>
     </row>
     <row r="260" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A260" s="16" t="str">
+      <c r="A260" s="11" t="str">
         <f>IF(B260&lt;&gt;"",COUNT($B$6:B260),"")</f>
         <v/>
       </c>
@@ -7882,7 +7912,7 @@
       <c r="O260" s="12"/>
     </row>
     <row r="261" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A261" s="16" t="str">
+      <c r="A261" s="11" t="str">
         <f>IF(B261&lt;&gt;"",COUNT($B$6:B261),"")</f>
         <v/>
       </c>
@@ -7908,7 +7938,7 @@
       <c r="O261" s="12"/>
     </row>
     <row r="262" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A262" s="16" t="str">
+      <c r="A262" s="11" t="str">
         <f>IF(B262&lt;&gt;"",COUNT($B$6:B262),"")</f>
         <v/>
       </c>
@@ -7934,7 +7964,7 @@
       <c r="O262" s="12"/>
     </row>
     <row r="263" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A263" s="16" t="str">
+      <c r="A263" s="11" t="str">
         <f>IF(B263&lt;&gt;"",COUNT($B$6:B263),"")</f>
         <v/>
       </c>
@@ -7960,7 +7990,7 @@
       <c r="O263" s="12"/>
     </row>
     <row r="264" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A264" s="16" t="str">
+      <c r="A264" s="11" t="str">
         <f>IF(B264&lt;&gt;"",COUNT($B$6:B264),"")</f>
         <v/>
       </c>
@@ -7986,7 +8016,7 @@
       <c r="O264" s="12"/>
     </row>
     <row r="265" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A265" s="16" t="str">
+      <c r="A265" s="11" t="str">
         <f>IF(B265&lt;&gt;"",COUNT($B$6:B265),"")</f>
         <v/>
       </c>
@@ -8012,7 +8042,7 @@
       <c r="O265" s="12"/>
     </row>
     <row r="266" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A266" s="16" t="str">
+      <c r="A266" s="11" t="str">
         <f>IF(B266&lt;&gt;"",COUNT($B$6:B266),"")</f>
         <v/>
       </c>
@@ -8038,7 +8068,7 @@
       <c r="O266" s="12"/>
     </row>
     <row r="267" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A267" s="16" t="str">
+      <c r="A267" s="11" t="str">
         <f>IF(B267&lt;&gt;"",COUNT($B$6:B267),"")</f>
         <v/>
       </c>
@@ -8064,7 +8094,7 @@
       <c r="O267" s="12"/>
     </row>
     <row r="268" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A268" s="16" t="str">
+      <c r="A268" s="11" t="str">
         <f>IF(B268&lt;&gt;"",COUNT($B$6:B268),"")</f>
         <v/>
       </c>
@@ -8090,7 +8120,7 @@
       <c r="O268" s="12"/>
     </row>
     <row r="269" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A269" s="16" t="str">
+      <c r="A269" s="11" t="str">
         <f>IF(B269&lt;&gt;"",COUNT($B$6:B269),"")</f>
         <v/>
       </c>
@@ -8116,7 +8146,7 @@
       <c r="O269" s="12"/>
     </row>
     <row r="270" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A270" s="16" t="str">
+      <c r="A270" s="11" t="str">
         <f>IF(B270&lt;&gt;"",COUNT($B$6:B270),"")</f>
         <v/>
       </c>
@@ -8142,7 +8172,7 @@
       <c r="O270" s="12"/>
     </row>
     <row r="271" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A271" s="16" t="str">
+      <c r="A271" s="11" t="str">
         <f>IF(B271&lt;&gt;"",COUNT($B$6:B271),"")</f>
         <v/>
       </c>
@@ -8168,7 +8198,7 @@
       <c r="O271" s="12"/>
     </row>
     <row r="272" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A272" s="16" t="str">
+      <c r="A272" s="11" t="str">
         <f>IF(B272&lt;&gt;"",COUNT($B$6:B272),"")</f>
         <v/>
       </c>
@@ -8194,7 +8224,7 @@
       <c r="O272" s="12"/>
     </row>
     <row r="273" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A273" s="16" t="str">
+      <c r="A273" s="11" t="str">
         <f>IF(B273&lt;&gt;"",COUNT($B$6:B273),"")</f>
         <v/>
       </c>
@@ -8220,7 +8250,7 @@
       <c r="O273" s="12"/>
     </row>
     <row r="274" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A274" s="16" t="str">
+      <c r="A274" s="11" t="str">
         <f>IF(B274&lt;&gt;"",COUNT($B$6:B274),"")</f>
         <v/>
       </c>
@@ -8246,7 +8276,7 @@
       <c r="O274" s="12"/>
     </row>
     <row r="275" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A275" s="16" t="str">
+      <c r="A275" s="11" t="str">
         <f>IF(B275&lt;&gt;"",COUNT($B$6:B275),"")</f>
         <v/>
       </c>
@@ -8272,7 +8302,7 @@
       <c r="O275" s="12"/>
     </row>
     <row r="276" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A276" s="16" t="str">
+      <c r="A276" s="11" t="str">
         <f>IF(B276&lt;&gt;"",COUNT($B$6:B276),"")</f>
         <v/>
       </c>
@@ -8298,7 +8328,7 @@
       <c r="O276" s="12"/>
     </row>
     <row r="277" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A277" s="16" t="str">
+      <c r="A277" s="11" t="str">
         <f>IF(B277&lt;&gt;"",COUNT($B$6:B277),"")</f>
         <v/>
       </c>
@@ -8324,7 +8354,7 @@
       <c r="O277" s="12"/>
     </row>
     <row r="278" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A278" s="16" t="str">
+      <c r="A278" s="11" t="str">
         <f>IF(B278&lt;&gt;"",COUNT($B$6:B278),"")</f>
         <v/>
       </c>
@@ -8350,7 +8380,7 @@
       <c r="O278" s="12"/>
     </row>
     <row r="279" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A279" s="16" t="str">
+      <c r="A279" s="11" t="str">
         <f>IF(B279&lt;&gt;"",COUNT($B$6:B279),"")</f>
         <v/>
       </c>
@@ -8376,7 +8406,7 @@
       <c r="O279" s="12"/>
     </row>
     <row r="280" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A280" s="16" t="str">
+      <c r="A280" s="11" t="str">
         <f>IF(B280&lt;&gt;"",COUNT($B$6:B280),"")</f>
         <v/>
       </c>
@@ -8402,7 +8432,7 @@
       <c r="O280" s="12"/>
     </row>
     <row r="281" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A281" s="16" t="str">
+      <c r="A281" s="11" t="str">
         <f>IF(B281&lt;&gt;"",COUNT($B$6:B281),"")</f>
         <v/>
       </c>
@@ -8428,7 +8458,7 @@
       <c r="O281" s="12"/>
     </row>
     <row r="282" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A282" s="16" t="str">
+      <c r="A282" s="11" t="str">
         <f>IF(B282&lt;&gt;"",COUNT($B$6:B282),"")</f>
         <v/>
       </c>
@@ -8454,7 +8484,7 @@
       <c r="O282" s="12"/>
     </row>
     <row r="283" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A283" s="16" t="str">
+      <c r="A283" s="11" t="str">
         <f>IF(B283&lt;&gt;"",COUNT($B$6:B283),"")</f>
         <v/>
       </c>
@@ -8480,7 +8510,7 @@
       <c r="O283" s="12"/>
     </row>
     <row r="284" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A284" s="16" t="str">
+      <c r="A284" s="11" t="str">
         <f>IF(B284&lt;&gt;"",COUNT($B$6:B284),"")</f>
         <v/>
       </c>
@@ -8506,7 +8536,7 @@
       <c r="O284" s="12"/>
     </row>
     <row r="285" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A285" s="16" t="str">
+      <c r="A285" s="11" t="str">
         <f>IF(B285&lt;&gt;"",COUNT($B$6:B285),"")</f>
         <v/>
       </c>
@@ -8532,7 +8562,7 @@
       <c r="O285" s="12"/>
     </row>
     <row r="286" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A286" s="16" t="str">
+      <c r="A286" s="11" t="str">
         <f>IF(B286&lt;&gt;"",COUNT($B$6:B286),"")</f>
         <v/>
       </c>
@@ -8558,7 +8588,7 @@
       <c r="O286" s="12"/>
     </row>
     <row r="287" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A287" s="16" t="str">
+      <c r="A287" s="11" t="str">
         <f>IF(B287&lt;&gt;"",COUNT($B$6:B287),"")</f>
         <v/>
       </c>
@@ -8584,7 +8614,7 @@
       <c r="O287" s="12"/>
     </row>
     <row r="288" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A288" s="16" t="str">
+      <c r="A288" s="11" t="str">
         <f>IF(B288&lt;&gt;"",COUNT($B$6:B288),"")</f>
         <v/>
       </c>
@@ -8610,7 +8640,7 @@
       <c r="O288" s="12"/>
     </row>
     <row r="289" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A289" s="16" t="str">
+      <c r="A289" s="11" t="str">
         <f>IF(B289&lt;&gt;"",COUNT($B$6:B289),"")</f>
         <v/>
       </c>
@@ -8636,7 +8666,7 @@
       <c r="O289" s="12"/>
     </row>
     <row r="290" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A290" s="16" t="str">
+      <c r="A290" s="11" t="str">
         <f>IF(B290&lt;&gt;"",COUNT($B$6:B290),"")</f>
         <v/>
       </c>
@@ -8662,7 +8692,7 @@
       <c r="O290" s="12"/>
     </row>
     <row r="291" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A291" s="16" t="str">
+      <c r="A291" s="11" t="str">
         <f>IF(B291&lt;&gt;"",COUNT($B$6:B291),"")</f>
         <v/>
       </c>
@@ -8688,7 +8718,7 @@
       <c r="O291" s="12"/>
     </row>
     <row r="292" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A292" s="16" t="str">
+      <c r="A292" s="11" t="str">
         <f>IF(B292&lt;&gt;"",COUNT($B$6:B292),"")</f>
         <v/>
       </c>
@@ -8714,7 +8744,7 @@
       <c r="O292" s="12"/>
     </row>
     <row r="293" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A293" s="16" t="str">
+      <c r="A293" s="11" t="str">
         <f>IF(B293&lt;&gt;"",COUNT($B$6:B293),"")</f>
         <v/>
       </c>
@@ -8740,7 +8770,7 @@
       <c r="O293" s="12"/>
     </row>
     <row r="294" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A294" s="16" t="str">
+      <c r="A294" s="11" t="str">
         <f>IF(B294&lt;&gt;"",COUNT($B$6:B294),"")</f>
         <v/>
       </c>
@@ -8766,7 +8796,7 @@
       <c r="O294" s="12"/>
     </row>
     <row r="295" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A295" s="16" t="str">
+      <c r="A295" s="11" t="str">
         <f>IF(B295&lt;&gt;"",COUNT($B$6:B295),"")</f>
         <v/>
       </c>
@@ -8792,7 +8822,7 @@
       <c r="O295" s="12"/>
     </row>
     <row r="296" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A296" s="16" t="str">
+      <c r="A296" s="11" t="str">
         <f>IF(B296&lt;&gt;"",COUNT($B$6:B296),"")</f>
         <v/>
       </c>
@@ -8818,7 +8848,7 @@
       <c r="O296" s="12"/>
     </row>
     <row r="297" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A297" s="16" t="str">
+      <c r="A297" s="11" t="str">
         <f>IF(B297&lt;&gt;"",COUNT($B$6:B297),"")</f>
         <v/>
       </c>
@@ -8844,7 +8874,7 @@
       <c r="O297" s="12"/>
     </row>
     <row r="298" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A298" s="16" t="str">
+      <c r="A298" s="11" t="str">
         <f>IF(B298&lt;&gt;"",COUNT($B$6:B298),"")</f>
         <v/>
       </c>
@@ -8870,7 +8900,7 @@
       <c r="O298" s="12"/>
     </row>
     <row r="299" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A299" s="16" t="str">
+      <c r="A299" s="11" t="str">
         <f>IF(B299&lt;&gt;"",COUNT($B$6:B299),"")</f>
         <v/>
       </c>
@@ -8896,7 +8926,7 @@
       <c r="O299" s="12"/>
     </row>
     <row r="300" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A300" s="16" t="str">
+      <c r="A300" s="11" t="str">
         <f>IF(B300&lt;&gt;"",COUNT($B$6:B300),"")</f>
         <v/>
       </c>
@@ -8922,7 +8952,7 @@
       <c r="O300" s="12"/>
     </row>
     <row r="301" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A301" s="16" t="str">
+      <c r="A301" s="11" t="str">
         <f>IF(B301&lt;&gt;"",COUNT($B$6:B301),"")</f>
         <v/>
       </c>
@@ -8948,7 +8978,7 @@
       <c r="O301" s="12"/>
     </row>
     <row r="302" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A302" s="16" t="str">
+      <c r="A302" s="11" t="str">
         <f>IF(B302&lt;&gt;"",COUNT($B$6:B302),"")</f>
         <v/>
       </c>
@@ -8974,7 +9004,7 @@
       <c r="O302" s="12"/>
     </row>
     <row r="303" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A303" s="16" t="str">
+      <c r="A303" s="11" t="str">
         <f>IF(B303&lt;&gt;"",COUNT($B$6:B303),"")</f>
         <v/>
       </c>
@@ -9000,7 +9030,7 @@
       <c r="O303" s="12"/>
     </row>
     <row r="304" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A304" s="16" t="str">
+      <c r="A304" s="11" t="str">
         <f>IF(B304&lt;&gt;"",COUNT($B$6:B304),"")</f>
         <v/>
       </c>
@@ -9026,7 +9056,7 @@
       <c r="O304" s="12"/>
     </row>
     <row r="305" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A305" s="16" t="str">
+      <c r="A305" s="11" t="str">
         <f>IF(B305&lt;&gt;"",COUNT($B$6:B305),"")</f>
         <v/>
       </c>
@@ -9052,7 +9082,7 @@
       <c r="O305" s="12"/>
     </row>
     <row r="306" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A306" s="16" t="str">
+      <c r="A306" s="11" t="str">
         <f>IF(B306&lt;&gt;"",COUNT($B$6:B306),"")</f>
         <v/>
       </c>
@@ -9078,7 +9108,7 @@
       <c r="O306" s="12"/>
     </row>
     <row r="307" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A307" s="16" t="str">
+      <c r="A307" s="11" t="str">
         <f>IF(B307&lt;&gt;"",COUNT($B$6:B307),"")</f>
         <v/>
       </c>
@@ -9104,7 +9134,7 @@
       <c r="O307" s="12"/>
     </row>
     <row r="308" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A308" s="16" t="str">
+      <c r="A308" s="11" t="str">
         <f>IF(B308&lt;&gt;"",COUNT($B$6:B308),"")</f>
         <v/>
       </c>
@@ -9130,7 +9160,7 @@
       <c r="O308" s="12"/>
     </row>
     <row r="309" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A309" s="16" t="str">
+      <c r="A309" s="11" t="str">
         <f>IF(B309&lt;&gt;"",COUNT($B$6:B309),"")</f>
         <v/>
       </c>
@@ -9156,7 +9186,7 @@
       <c r="O309" s="12"/>
     </row>
     <row r="310" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A310" s="16" t="str">
+      <c r="A310" s="11" t="str">
         <f>IF(B310&lt;&gt;"",COUNT($B$6:B310),"")</f>
         <v/>
       </c>
@@ -9182,7 +9212,7 @@
       <c r="O310" s="12"/>
     </row>
     <row r="311" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A311" s="16" t="str">
+      <c r="A311" s="11" t="str">
         <f>IF(B311&lt;&gt;"",COUNT($B$6:B311),"")</f>
         <v/>
       </c>
@@ -9208,7 +9238,7 @@
       <c r="O311" s="12"/>
     </row>
     <row r="312" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A312" s="16" t="str">
+      <c r="A312" s="11" t="str">
         <f>IF(B312&lt;&gt;"",COUNT($B$6:B312),"")</f>
         <v/>
       </c>
@@ -9234,7 +9264,7 @@
       <c r="O312" s="12"/>
     </row>
     <row r="313" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A313" s="16" t="str">
+      <c r="A313" s="11" t="str">
         <f>IF(B313&lt;&gt;"",COUNT($B$6:B313),"")</f>
         <v/>
       </c>
@@ -9260,7 +9290,7 @@
       <c r="O313" s="12"/>
     </row>
     <row r="314" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A314" s="16" t="str">
+      <c r="A314" s="11" t="str">
         <f>IF(B314&lt;&gt;"",COUNT($B$6:B314),"")</f>
         <v/>
       </c>
@@ -9286,7 +9316,7 @@
       <c r="O314" s="12"/>
     </row>
     <row r="315" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A315" s="16" t="str">
+      <c r="A315" s="11" t="str">
         <f>IF(B315&lt;&gt;"",COUNT($B$6:B315),"")</f>
         <v/>
       </c>
@@ -9312,7 +9342,7 @@
       <c r="O315" s="12"/>
     </row>
     <row r="316" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A316" s="16" t="str">
+      <c r="A316" s="11" t="str">
         <f>IF(B316&lt;&gt;"",COUNT($B$6:B316),"")</f>
         <v/>
       </c>
@@ -9338,7 +9368,7 @@
       <c r="O316" s="12"/>
     </row>
     <row r="317" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A317" s="16" t="str">
+      <c r="A317" s="11" t="str">
         <f>IF(B317&lt;&gt;"",COUNT($B$6:B317),"")</f>
         <v/>
       </c>
@@ -9364,7 +9394,7 @@
       <c r="O317" s="12"/>
     </row>
     <row r="318" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A318" s="16" t="str">
+      <c r="A318" s="11" t="str">
         <f>IF(B318&lt;&gt;"",COUNT($B$6:B318),"")</f>
         <v/>
       </c>
@@ -9390,7 +9420,7 @@
       <c r="O318" s="12"/>
     </row>
     <row r="319" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A319" s="16" t="str">
+      <c r="A319" s="11" t="str">
         <f>IF(B319&lt;&gt;"",COUNT($B$6:B319),"")</f>
         <v/>
       </c>
@@ -9416,7 +9446,7 @@
       <c r="O319" s="12"/>
     </row>
     <row r="320" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A320" s="16" t="str">
+      <c r="A320" s="11" t="str">
         <f>IF(B320&lt;&gt;"",COUNT($B$6:B320),"")</f>
         <v/>
       </c>
@@ -9442,7 +9472,7 @@
       <c r="O320" s="12"/>
     </row>
     <row r="321" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A321" s="16" t="str">
+      <c r="A321" s="11" t="str">
         <f>IF(B321&lt;&gt;"",COUNT($B$6:B321),"")</f>
         <v/>
       </c>
@@ -9468,7 +9498,7 @@
       <c r="O321" s="12"/>
     </row>
     <row r="322" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A322" s="16" t="str">
+      <c r="A322" s="11" t="str">
         <f>IF(B322&lt;&gt;"",COUNT($B$6:B322),"")</f>
         <v/>
       </c>
@@ -9494,7 +9524,7 @@
       <c r="O322" s="12"/>
     </row>
     <row r="323" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A323" s="16" t="str">
+      <c r="A323" s="11" t="str">
         <f>IF(B323&lt;&gt;"",COUNT($B$6:B323),"")</f>
         <v/>
       </c>
@@ -9520,7 +9550,7 @@
       <c r="O323" s="12"/>
     </row>
     <row r="324" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A324" s="16" t="str">
+      <c r="A324" s="11" t="str">
         <f>IF(B324&lt;&gt;"",COUNT($B$6:B324),"")</f>
         <v/>
       </c>
@@ -9546,7 +9576,7 @@
       <c r="O324" s="12"/>
     </row>
     <row r="325" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A325" s="16" t="str">
+      <c r="A325" s="11" t="str">
         <f>IF(B325&lt;&gt;"",COUNT($B$6:B325),"")</f>
         <v/>
       </c>
@@ -9572,7 +9602,7 @@
       <c r="O325" s="12"/>
     </row>
     <row r="326" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A326" s="16" t="str">
+      <c r="A326" s="11" t="str">
         <f>IF(B326&lt;&gt;"",COUNT($B$6:B326),"")</f>
         <v/>
       </c>
@@ -9598,7 +9628,7 @@
       <c r="O326" s="12"/>
     </row>
     <row r="327" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A327" s="16" t="str">
+      <c r="A327" s="11" t="str">
         <f>IF(B327&lt;&gt;"",COUNT($B$6:B327),"")</f>
         <v/>
       </c>
@@ -9624,7 +9654,7 @@
       <c r="O327" s="12"/>
     </row>
     <row r="328" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A328" s="16" t="str">
+      <c r="A328" s="11" t="str">
         <f>IF(B328&lt;&gt;"",COUNT($B$6:B328),"")</f>
         <v/>
       </c>
@@ -9650,7 +9680,7 @@
       <c r="O328" s="12"/>
     </row>
     <row r="329" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A329" s="16" t="str">
+      <c r="A329" s="11" t="str">
         <f>IF(B329&lt;&gt;"",COUNT($B$6:B329),"")</f>
         <v/>
       </c>
@@ -9676,7 +9706,7 @@
       <c r="O329" s="12"/>
     </row>
     <row r="330" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A330" s="16" t="str">
+      <c r="A330" s="11" t="str">
         <f>IF(B330&lt;&gt;"",COUNT($B$6:B330),"")</f>
         <v/>
       </c>
@@ -9702,7 +9732,7 @@
       <c r="O330" s="12"/>
     </row>
     <row r="331" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A331" s="16" t="str">
+      <c r="A331" s="11" t="str">
         <f>IF(B331&lt;&gt;"",COUNT($B$6:B331),"")</f>
         <v/>
       </c>
@@ -9728,7 +9758,7 @@
       <c r="O331" s="12"/>
     </row>
     <row r="332" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A332" s="16" t="str">
+      <c r="A332" s="11" t="str">
         <f>IF(B332&lt;&gt;"",COUNT($B$6:B332),"")</f>
         <v/>
       </c>
@@ -9754,7 +9784,7 @@
       <c r="O332" s="12"/>
     </row>
     <row r="333" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A333" s="16" t="str">
+      <c r="A333" s="11" t="str">
         <f>IF(B333&lt;&gt;"",COUNT($B$6:B333),"")</f>
         <v/>
       </c>
@@ -9780,7 +9810,7 @@
       <c r="O333" s="12"/>
     </row>
     <row r="334" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A334" s="16" t="str">
+      <c r="A334" s="11" t="str">
         <f>IF(B334&lt;&gt;"",COUNT($B$6:B334),"")</f>
         <v/>
       </c>
@@ -9806,7 +9836,7 @@
       <c r="O334" s="12"/>
     </row>
     <row r="335" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A335" s="16" t="str">
+      <c r="A335" s="11" t="str">
         <f>IF(B335&lt;&gt;"",COUNT($B$6:B335),"")</f>
         <v/>
       </c>
@@ -9832,7 +9862,7 @@
       <c r="O335" s="12"/>
     </row>
     <row r="336" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A336" s="16" t="str">
+      <c r="A336" s="11" t="str">
         <f>IF(B336&lt;&gt;"",COUNT($B$6:B336),"")</f>
         <v/>
       </c>
@@ -9858,7 +9888,7 @@
       <c r="O336" s="12"/>
     </row>
     <row r="337" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A337" s="16" t="str">
+      <c r="A337" s="11" t="str">
         <f>IF(B337&lt;&gt;"",COUNT($B$6:B337),"")</f>
         <v/>
       </c>
@@ -9884,7 +9914,7 @@
       <c r="O337" s="12"/>
     </row>
     <row r="338" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A338" s="16" t="str">
+      <c r="A338" s="11" t="str">
         <f>IF(B338&lt;&gt;"",COUNT($B$6:B338),"")</f>
         <v/>
       </c>
@@ -9910,7 +9940,7 @@
       <c r="O338" s="12"/>
     </row>
     <row r="339" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A339" s="16" t="str">
+      <c r="A339" s="11" t="str">
         <f>IF(B339&lt;&gt;"",COUNT($B$6:B339),"")</f>
         <v/>
       </c>
@@ -9936,7 +9966,7 @@
       <c r="O339" s="12"/>
     </row>
     <row r="340" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A340" s="16" t="str">
+      <c r="A340" s="11" t="str">
         <f>IF(B340&lt;&gt;"",COUNT($B$6:B340),"")</f>
         <v/>
       </c>
@@ -9962,7 +9992,7 @@
       <c r="O340" s="12"/>
     </row>
     <row r="341" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A341" s="16" t="str">
+      <c r="A341" s="11" t="str">
         <f>IF(B341&lt;&gt;"",COUNT($B$6:B341),"")</f>
         <v/>
       </c>
@@ -9988,7 +10018,7 @@
       <c r="O341" s="12"/>
     </row>
     <row r="342" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A342" s="16" t="str">
+      <c r="A342" s="11" t="str">
         <f>IF(B342&lt;&gt;"",COUNT($B$6:B342),"")</f>
         <v/>
       </c>
@@ -10014,7 +10044,7 @@
       <c r="O342" s="12"/>
     </row>
     <row r="343" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A343" s="16" t="str">
+      <c r="A343" s="11" t="str">
         <f>IF(B343&lt;&gt;"",COUNT($B$6:B343),"")</f>
         <v/>
       </c>
@@ -10040,7 +10070,7 @@
       <c r="O343" s="12"/>
     </row>
     <row r="344" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A344" s="16" t="str">
+      <c r="A344" s="11" t="str">
         <f>IF(B344&lt;&gt;"",COUNT($B$6:B344),"")</f>
         <v/>
       </c>
@@ -10066,7 +10096,7 @@
       <c r="O344" s="12"/>
     </row>
     <row r="345" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A345" s="16" t="str">
+      <c r="A345" s="11" t="str">
         <f>IF(B345&lt;&gt;"",COUNT($B$6:B345),"")</f>
         <v/>
       </c>
@@ -10092,7 +10122,7 @@
       <c r="O345" s="12"/>
     </row>
     <row r="346" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A346" s="16" t="str">
+      <c r="A346" s="11" t="str">
         <f>IF(B346&lt;&gt;"",COUNT($B$6:B346),"")</f>
         <v/>
       </c>
@@ -10118,7 +10148,7 @@
       <c r="O346" s="12"/>
     </row>
     <row r="347" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A347" s="16" t="str">
+      <c r="A347" s="11" t="str">
         <f>IF(B347&lt;&gt;"",COUNT($B$6:B347),"")</f>
         <v/>
       </c>
@@ -10144,7 +10174,7 @@
       <c r="O347" s="12"/>
     </row>
     <row r="348" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A348" s="16" t="str">
+      <c r="A348" s="11" t="str">
         <f>IF(B348&lt;&gt;"",COUNT($B$6:B348),"")</f>
         <v/>
       </c>
@@ -10170,7 +10200,7 @@
       <c r="O348" s="12"/>
     </row>
     <row r="349" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A349" s="16" t="str">
+      <c r="A349" s="11" t="str">
         <f>IF(B349&lt;&gt;"",COUNT($B$6:B349),"")</f>
         <v/>
       </c>
@@ -10196,7 +10226,7 @@
       <c r="O349" s="12"/>
     </row>
     <row r="350" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A350" s="16" t="str">
+      <c r="A350" s="11" t="str">
         <f>IF(B350&lt;&gt;"",COUNT($B$6:B350),"")</f>
         <v/>
       </c>
@@ -10222,7 +10252,7 @@
       <c r="O350" s="12"/>
     </row>
     <row r="351" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A351" s="16" t="str">
+      <c r="A351" s="11" t="str">
         <f>IF(B351&lt;&gt;"",COUNT($B$6:B351),"")</f>
         <v/>
       </c>
@@ -10248,7 +10278,7 @@
       <c r="O351" s="12"/>
     </row>
     <row r="352" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A352" s="16" t="str">
+      <c r="A352" s="11" t="str">
         <f>IF(B352&lt;&gt;"",COUNT($B$6:B352),"")</f>
         <v/>
       </c>
@@ -10274,7 +10304,7 @@
       <c r="O352" s="12"/>
     </row>
     <row r="353" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A353" s="16" t="str">
+      <c r="A353" s="11" t="str">
         <f>IF(B353&lt;&gt;"",COUNT($B$6:B353),"")</f>
         <v/>
       </c>
@@ -10300,7 +10330,7 @@
       <c r="O353" s="12"/>
     </row>
     <row r="354" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A354" s="16" t="str">
+      <c r="A354" s="11" t="str">
         <f>IF(B354&lt;&gt;"",COUNT($B$6:B354),"")</f>
         <v/>
       </c>
@@ -10326,7 +10356,7 @@
       <c r="O354" s="12"/>
     </row>
     <row r="355" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A355" s="16" t="str">
+      <c r="A355" s="11" t="str">
         <f>IF(B355&lt;&gt;"",COUNT($B$6:B355),"")</f>
         <v/>
       </c>
@@ -10352,7 +10382,7 @@
       <c r="O355" s="12"/>
     </row>
     <row r="356" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A356" s="16" t="str">
+      <c r="A356" s="11" t="str">
         <f>IF(B356&lt;&gt;"",COUNT($B$6:B356),"")</f>
         <v/>
       </c>
@@ -10378,7 +10408,7 @@
       <c r="O356" s="12"/>
     </row>
     <row r="357" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A357" s="16" t="str">
+      <c r="A357" s="11" t="str">
         <f>IF(B357&lt;&gt;"",COUNT($B$6:B357),"")</f>
         <v/>
       </c>
@@ -10404,7 +10434,7 @@
       <c r="O357" s="12"/>
     </row>
     <row r="358" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A358" s="16" t="str">
+      <c r="A358" s="11" t="str">
         <f>IF(B358&lt;&gt;"",COUNT($B$6:B358),"")</f>
         <v/>
       </c>
@@ -10430,7 +10460,7 @@
       <c r="O358" s="12"/>
     </row>
     <row r="359" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A359" s="16" t="str">
+      <c r="A359" s="11" t="str">
         <f>IF(B359&lt;&gt;"",COUNT($B$6:B359),"")</f>
         <v/>
       </c>
@@ -10456,7 +10486,7 @@
       <c r="O359" s="12"/>
     </row>
     <row r="360" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A360" s="16" t="str">
+      <c r="A360" s="11" t="str">
         <f>IF(B360&lt;&gt;"",COUNT($B$6:B360),"")</f>
         <v/>
       </c>
@@ -10482,7 +10512,7 @@
       <c r="O360" s="12"/>
     </row>
     <row r="361" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A361" s="16" t="str">
+      <c r="A361" s="11" t="str">
         <f>IF(B361&lt;&gt;"",COUNT($B$6:B361),"")</f>
         <v/>
       </c>
@@ -10508,7 +10538,7 @@
       <c r="O361" s="12"/>
     </row>
     <row r="362" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A362" s="16" t="str">
+      <c r="A362" s="11" t="str">
         <f>IF(B362&lt;&gt;"",COUNT($B$6:B362),"")</f>
         <v/>
       </c>
@@ -10534,7 +10564,7 @@
       <c r="O362" s="12"/>
     </row>
     <row r="363" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A363" s="16" t="str">
+      <c r="A363" s="11" t="str">
         <f>IF(B363&lt;&gt;"",COUNT($B$6:B363),"")</f>
         <v/>
       </c>
@@ -10560,7 +10590,7 @@
       <c r="O363" s="12"/>
     </row>
     <row r="364" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A364" s="16" t="str">
+      <c r="A364" s="11" t="str">
         <f>IF(B364&lt;&gt;"",COUNT($B$6:B364),"")</f>
         <v/>
       </c>
@@ -10586,7 +10616,7 @@
       <c r="O364" s="12"/>
     </row>
     <row r="365" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A365" s="16" t="str">
+      <c r="A365" s="11" t="str">
         <f>IF(B365&lt;&gt;"",COUNT($B$6:B365),"")</f>
         <v/>
       </c>
@@ -10612,7 +10642,7 @@
       <c r="O365" s="12"/>
     </row>
     <row r="366" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A366" s="16" t="str">
+      <c r="A366" s="11" t="str">
         <f>IF(B366&lt;&gt;"",COUNT($B$6:B366),"")</f>
         <v/>
       </c>
@@ -10638,7 +10668,7 @@
       <c r="O366" s="12"/>
     </row>
     <row r="367" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A367" s="16" t="str">
+      <c r="A367" s="11" t="str">
         <f>IF(B367&lt;&gt;"",COUNT($B$6:B367),"")</f>
         <v/>
       </c>
@@ -10664,7 +10694,7 @@
       <c r="O367" s="12"/>
     </row>
     <row r="368" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A368" s="16" t="str">
+      <c r="A368" s="11" t="str">
         <f>IF(B368&lt;&gt;"",COUNT($B$6:B368),"")</f>
         <v/>
       </c>
@@ -10690,7 +10720,7 @@
       <c r="O368" s="12"/>
     </row>
     <row r="369" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A369" s="16" t="str">
+      <c r="A369" s="11" t="str">
         <f>IF(B369&lt;&gt;"",COUNT($B$6:B369),"")</f>
         <v/>
       </c>
@@ -10716,7 +10746,7 @@
       <c r="O369" s="12"/>
     </row>
     <row r="370" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A370" s="16" t="str">
+      <c r="A370" s="11" t="str">
         <f>IF(B370&lt;&gt;"",COUNT($B$6:B370),"")</f>
         <v/>
       </c>
@@ -10742,7 +10772,7 @@
       <c r="O370" s="12"/>
     </row>
     <row r="371" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A371" s="16" t="str">
+      <c r="A371" s="11" t="str">
         <f>IF(B371&lt;&gt;"",COUNT($B$6:B371),"")</f>
         <v/>
       </c>
@@ -10768,7 +10798,7 @@
       <c r="O371" s="12"/>
     </row>
     <row r="372" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A372" s="16" t="str">
+      <c r="A372" s="11" t="str">
         <f>IF(B372&lt;&gt;"",COUNT($B$6:B372),"")</f>
         <v/>
       </c>
@@ -10794,7 +10824,7 @@
       <c r="O372" s="12"/>
     </row>
     <row r="373" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A373" s="16" t="str">
+      <c r="A373" s="11" t="str">
         <f>IF(B373&lt;&gt;"",COUNT($B$6:B373),"")</f>
         <v/>
       </c>
@@ -10820,7 +10850,7 @@
       <c r="O373" s="12"/>
     </row>
     <row r="374" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A374" s="16" t="str">
+      <c r="A374" s="11" t="str">
         <f>IF(B374&lt;&gt;"",COUNT($B$6:B374),"")</f>
         <v/>
       </c>
@@ -10846,7 +10876,7 @@
       <c r="O374" s="12"/>
     </row>
     <row r="375" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A375" s="16" t="str">
+      <c r="A375" s="11" t="str">
         <f>IF(B375&lt;&gt;"",COUNT($B$6:B375),"")</f>
         <v/>
       </c>
@@ -10872,7 +10902,7 @@
       <c r="O375" s="12"/>
     </row>
     <row r="376" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A376" s="16" t="str">
+      <c r="A376" s="11" t="str">
         <f>IF(B376&lt;&gt;"",COUNT($B$6:B376),"")</f>
         <v/>
       </c>
@@ -10898,7 +10928,7 @@
       <c r="O376" s="12"/>
     </row>
     <row r="377" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A377" s="16" t="str">
+      <c r="A377" s="11" t="str">
         <f>IF(B377&lt;&gt;"",COUNT($B$6:B377),"")</f>
         <v/>
       </c>
@@ -10924,7 +10954,7 @@
       <c r="O377" s="12"/>
     </row>
     <row r="378" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A378" s="16" t="str">
+      <c r="A378" s="11" t="str">
         <f>IF(B378&lt;&gt;"",COUNT($B$6:B378),"")</f>
         <v/>
       </c>
@@ -10950,7 +10980,7 @@
       <c r="O378" s="12"/>
     </row>
     <row r="379" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A379" s="16" t="str">
+      <c r="A379" s="11" t="str">
         <f>IF(B379&lt;&gt;"",COUNT($B$6:B379),"")</f>
         <v/>
       </c>
@@ -10976,7 +11006,7 @@
       <c r="O379" s="12"/>
     </row>
     <row r="380" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A380" s="16" t="str">
+      <c r="A380" s="11" t="str">
         <f>IF(B380&lt;&gt;"",COUNT($B$6:B380),"")</f>
         <v/>
       </c>
@@ -11002,7 +11032,7 @@
       <c r="O380" s="12"/>
     </row>
     <row r="381" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A381" s="16" t="str">
+      <c r="A381" s="11" t="str">
         <f>IF(B381&lt;&gt;"",COUNT($B$6:B381),"")</f>
         <v/>
       </c>
@@ -11028,7 +11058,7 @@
       <c r="O381" s="12"/>
     </row>
     <row r="382" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A382" s="16" t="str">
+      <c r="A382" s="11" t="str">
         <f>IF(B382&lt;&gt;"",COUNT($B$6:B382),"")</f>
         <v/>
       </c>
@@ -11054,7 +11084,7 @@
       <c r="O382" s="12"/>
     </row>
     <row r="383" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A383" s="16" t="str">
+      <c r="A383" s="11" t="str">
         <f>IF(B383&lt;&gt;"",COUNT($B$6:B383),"")</f>
         <v/>
       </c>
@@ -11080,7 +11110,7 @@
       <c r="O383" s="12"/>
     </row>
     <row r="384" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A384" s="16" t="str">
+      <c r="A384" s="11" t="str">
         <f>IF(B384&lt;&gt;"",COUNT($B$6:B384),"")</f>
         <v/>
       </c>
@@ -11106,7 +11136,7 @@
       <c r="O384" s="12"/>
     </row>
     <row r="385" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A385" s="16" t="str">
+      <c r="A385" s="11" t="str">
         <f>IF(B385&lt;&gt;"",COUNT($B$6:B385),"")</f>
         <v/>
       </c>
@@ -11132,7 +11162,7 @@
       <c r="O385" s="12"/>
     </row>
     <row r="386" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A386" s="16" t="str">
+      <c r="A386" s="11" t="str">
         <f>IF(B386&lt;&gt;"",COUNT($B$6:B386),"")</f>
         <v/>
       </c>
@@ -11158,7 +11188,7 @@
       <c r="O386" s="12"/>
     </row>
     <row r="387" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A387" s="16" t="str">
+      <c r="A387" s="11" t="str">
         <f>IF(B387&lt;&gt;"",COUNT($B$6:B387),"")</f>
         <v/>
       </c>
@@ -11184,7 +11214,7 @@
       <c r="O387" s="12"/>
     </row>
     <row r="388" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A388" s="16" t="str">
+      <c r="A388" s="11" t="str">
         <f>IF(B388&lt;&gt;"",COUNT($B$6:B388),"")</f>
         <v/>
       </c>
@@ -11210,7 +11240,7 @@
       <c r="O388" s="12"/>
     </row>
     <row r="389" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A389" s="16" t="str">
+      <c r="A389" s="11" t="str">
         <f>IF(B389&lt;&gt;"",COUNT($B$6:B389),"")</f>
         <v/>
       </c>
@@ -11236,7 +11266,7 @@
       <c r="O389" s="12"/>
     </row>
     <row r="390" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A390" s="16" t="str">
+      <c r="A390" s="11" t="str">
         <f>IF(B390&lt;&gt;"",COUNT($B$6:B390),"")</f>
         <v/>
       </c>
@@ -11262,7 +11292,7 @@
       <c r="O390" s="12"/>
     </row>
     <row r="391" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A391" s="16" t="str">
+      <c r="A391" s="11" t="str">
         <f>IF(B391&lt;&gt;"",COUNT($B$6:B391),"")</f>
         <v/>
       </c>
@@ -11288,7 +11318,7 @@
       <c r="O391" s="12"/>
     </row>
     <row r="392" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A392" s="16" t="str">
+      <c r="A392" s="11" t="str">
         <f>IF(B392&lt;&gt;"",COUNT($B$6:B392),"")</f>
         <v/>
       </c>
@@ -11314,7 +11344,7 @@
       <c r="O392" s="12"/>
     </row>
     <row r="393" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A393" s="16" t="str">
+      <c r="A393" s="11" t="str">
         <f>IF(B393&lt;&gt;"",COUNT($B$6:B393),"")</f>
         <v/>
       </c>
@@ -11340,7 +11370,7 @@
       <c r="O393" s="12"/>
     </row>
     <row r="394" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A394" s="16" t="str">
+      <c r="A394" s="11" t="str">
         <f>IF(B394&lt;&gt;"",COUNT($B$6:B394),"")</f>
         <v/>
       </c>
@@ -11366,7 +11396,7 @@
       <c r="O394" s="12"/>
     </row>
     <row r="395" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A395" s="16" t="str">
+      <c r="A395" s="11" t="str">
         <f>IF(B395&lt;&gt;"",COUNT($B$6:B395),"")</f>
         <v/>
       </c>
@@ -11392,7 +11422,7 @@
       <c r="O395" s="12"/>
     </row>
     <row r="396" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A396" s="16" t="str">
+      <c r="A396" s="11" t="str">
         <f>IF(B396&lt;&gt;"",COUNT($B$6:B396),"")</f>
         <v/>
       </c>
@@ -11418,7 +11448,7 @@
       <c r="O396" s="12"/>
     </row>
     <row r="397" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A397" s="16" t="str">
+      <c r="A397" s="11" t="str">
         <f>IF(B397&lt;&gt;"",COUNT($B$6:B397),"")</f>
         <v/>
       </c>
@@ -11444,7 +11474,7 @@
       <c r="O397" s="12"/>
     </row>
     <row r="398" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A398" s="16" t="str">
+      <c r="A398" s="11" t="str">
         <f>IF(B398&lt;&gt;"",COUNT($B$6:B398),"")</f>
         <v/>
       </c>
@@ -11470,7 +11500,7 @@
       <c r="O398" s="12"/>
     </row>
     <row r="399" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A399" s="16" t="str">
+      <c r="A399" s="11" t="str">
         <f>IF(B399&lt;&gt;"",COUNT($B$6:B399),"")</f>
         <v/>
       </c>
@@ -11496,7 +11526,7 @@
       <c r="O399" s="12"/>
     </row>
     <row r="400" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A400" s="16" t="str">
+      <c r="A400" s="11" t="str">
         <f>IF(B400&lt;&gt;"",COUNT($B$6:B400),"")</f>
         <v/>
       </c>
@@ -11522,7 +11552,7 @@
       <c r="O400" s="12"/>
     </row>
     <row r="401" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A401" s="16" t="str">
+      <c r="A401" s="11" t="str">
         <f>IF(B401&lt;&gt;"",COUNT($B$6:B401),"")</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Updated Excel File Day 12
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{294D1D48-5CFD-4052-8CA3-3B0446DB37C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8591DA6-0D8F-43B9-A6F1-E759872AE243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -257,6 +257,9 @@
   </si>
   <si>
     <t>I am not getting time to work on myself. I have to change myself.</t>
+  </si>
+  <si>
+    <t>I have fever today. It's tough for me to do anything today.</t>
   </si>
 </sst>
 </file>
@@ -1567,38 +1570,63 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="11" t="str">
+    <row r="17" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="11">
         <f>IF(B17&lt;&gt;"",COUNT($B$6:B17),"")</f>
-        <v/>
-      </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="10" t="str">
+        <v>12</v>
+      </c>
+      <c r="B17" s="8">
+        <v>46263</v>
+      </c>
+      <c r="C17" s="9">
+        <v>480</v>
+      </c>
+      <c r="D17" s="9">
+        <v>15</v>
+      </c>
+      <c r="E17" s="9">
+        <v>40</v>
+      </c>
+      <c r="F17" s="9">
+        <v>50</v>
+      </c>
+      <c r="G17" s="9">
+        <v>0</v>
+      </c>
+      <c r="H17" s="9">
+        <v>0</v>
+      </c>
+      <c r="I17" s="9">
+        <v>100</v>
+      </c>
+      <c r="J17" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K17" s="10" t="str">
+        <v>685</v>
+      </c>
+      <c r="K17" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="12"/>
+        <v>755</v>
+      </c>
+      <c r="L17" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="N17" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O17" s="12" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18" s="11" t="str">
-        <f>IF(B18&lt;&gt;"",COUNT($B$6:B18),"")</f>
-        <v/>
-      </c>
-      <c r="B18" s="8"/>
+      <c r="A18" s="11">
+        <v>13</v>
+      </c>
+      <c r="B18" s="8">
+        <v>46264</v>
+      </c>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
       <c r="E18" s="9"/>

</xml_diff>

<commit_message>
Updated Excel Data Day 13
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8591DA6-0D8F-43B9-A6F1-E759872AE243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE9142F8-4368-4C8C-A7C6-33B3042DC7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -260,6 +260,9 @@
   </si>
   <si>
     <t>I have fever today. It's tough for me to do anything today.</t>
+  </si>
+  <si>
+    <t>Couldn't do anything productive because of powercut today.</t>
   </si>
 </sst>
 </file>
@@ -1620,32 +1623,54 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="11">
         <v>13</v>
       </c>
       <c r="B18" s="8">
         <v>46264</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="10" t="str">
+      <c r="C18" s="9">
+        <v>360</v>
+      </c>
+      <c r="D18" s="9">
+        <v>10</v>
+      </c>
+      <c r="E18" s="9">
+        <v>30</v>
+      </c>
+      <c r="F18" s="9">
+        <v>40</v>
+      </c>
+      <c r="G18" s="9">
+        <v>0</v>
+      </c>
+      <c r="H18" s="9">
+        <v>0</v>
+      </c>
+      <c r="I18" s="9">
+        <v>120</v>
+      </c>
+      <c r="J18" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K18" s="10" t="str">
+        <v>560</v>
+      </c>
+      <c r="K18" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="12"/>
+        <v>880</v>
+      </c>
+      <c r="L18" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M18" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="N18" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O18" s="12" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 14
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE9142F8-4368-4C8C-A7C6-33B3042DC7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A437F03-9842-4685-BDDE-68472254785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -263,6 +263,9 @@
   </si>
   <si>
     <t>Couldn't do anything productive because of powercut today.</t>
+  </si>
+  <si>
+    <t>Need more Guts so that I can speak english during class</t>
   </si>
 </sst>
 </file>
@@ -1672,31 +1675,54 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="11" t="str">
-        <f>IF(B19&lt;&gt;"",COUNT($B$6:B19),"")</f>
-        <v/>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="10" t="str">
+    <row r="19" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="11">
+        <v>14</v>
+      </c>
+      <c r="B19" s="8">
+        <v>46265</v>
+      </c>
+      <c r="C19" s="9">
+        <v>420</v>
+      </c>
+      <c r="D19" s="9">
+        <v>20</v>
+      </c>
+      <c r="E19" s="9">
+        <v>25</v>
+      </c>
+      <c r="F19" s="9">
+        <v>55</v>
+      </c>
+      <c r="G19" s="9">
+        <v>200</v>
+      </c>
+      <c r="H19" s="9">
+        <v>4</v>
+      </c>
+      <c r="I19" s="9">
+        <v>45</v>
+      </c>
+      <c r="J19" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K19" s="10" t="str">
+        <v>765</v>
+      </c>
+      <c r="K19" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="12"/>
+        <v>675</v>
+      </c>
+      <c r="L19" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N19" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O19" s="12" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 15
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A437F03-9842-4685-BDDE-68472254785E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85C5C6C-7C84-47BD-ADF5-B1BA0F68A4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -266,6 +266,9 @@
   </si>
   <si>
     <t>Need more Guts so that I can speak english during class</t>
+  </si>
+  <si>
+    <t>I missed my first lecture because of my friend. He was very late.</t>
   </si>
 </sst>
 </file>
@@ -1724,31 +1727,54 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="11" t="str">
-        <f>IF(B20&lt;&gt;"",COUNT($B$6:B20),"")</f>
-        <v/>
-      </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="10" t="str">
+    <row r="20" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="11">
+        <v>15</v>
+      </c>
+      <c r="B20" s="8">
+        <v>46266</v>
+      </c>
+      <c r="C20" s="9">
+        <v>375</v>
+      </c>
+      <c r="D20" s="9">
+        <v>10</v>
+      </c>
+      <c r="E20" s="9">
+        <v>20</v>
+      </c>
+      <c r="F20" s="9">
+        <v>120</v>
+      </c>
+      <c r="G20" s="9">
+        <v>200</v>
+      </c>
+      <c r="H20" s="9">
+        <v>4</v>
+      </c>
+      <c r="I20" s="9">
+        <v>200</v>
+      </c>
+      <c r="J20" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K20" s="10" t="str">
+        <v>925</v>
+      </c>
+      <c r="K20" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="12"/>
+        <v>515</v>
+      </c>
+      <c r="L20" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="N20" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O20" s="12" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel Data Day 16
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F85C5C6C-7C84-47BD-ADF5-B1BA0F68A4A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F838514A-22F5-4C9C-832A-D19E73428E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t>I missed my first lecture because of my friend. He was very late.</t>
+  </si>
+  <si>
+    <t>I need to work harder. So, that I can improve myself.</t>
   </si>
 </sst>
 </file>
@@ -1776,31 +1779,54 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="11" t="str">
-        <f>IF(B21&lt;&gt;"",COUNT($B$6:B21),"")</f>
-        <v/>
-      </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="9"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="10" t="str">
+    <row r="21" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="11">
+        <v>16</v>
+      </c>
+      <c r="B21" s="8">
+        <v>46267</v>
+      </c>
+      <c r="C21" s="9">
+        <v>390</v>
+      </c>
+      <c r="D21" s="9">
+        <v>15</v>
+      </c>
+      <c r="E21" s="9">
+        <v>40</v>
+      </c>
+      <c r="F21" s="9">
+        <v>100</v>
+      </c>
+      <c r="G21" s="9">
+        <v>300</v>
+      </c>
+      <c r="H21" s="9">
+        <v>5</v>
+      </c>
+      <c r="I21" s="9">
+        <v>40</v>
+      </c>
+      <c r="J21" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K21" s="10" t="str">
+        <v>885</v>
+      </c>
+      <c r="K21" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="12"/>
+        <v>555</v>
+      </c>
+      <c r="L21" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="M21" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="N21" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="O21" s="12" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="str">

</xml_diff>

<commit_message>
Updated Excel File Day 17
</commit_message>
<xml_diff>
--- a/12612197.xlsx
+++ b/12612197.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding Journey\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F838514A-22F5-4C9C-832A-D19E73428E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E109298A-9EEE-4A91-980C-DFE85C8CFA64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -272,6 +272,9 @@
   </si>
   <si>
     <t>I need to work harder. So, that I can improve myself.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I need to have better control over my emotions. </t>
   </si>
 </sst>
 </file>
@@ -1828,31 +1831,54 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A22" s="11" t="str">
-        <f>IF(B22&lt;&gt;"",COUNT($B$6:B22),"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="9"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="9"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="10" t="str">
+    <row r="22" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="11">
+        <v>17</v>
+      </c>
+      <c r="B22" s="8">
+        <v>46268</v>
+      </c>
+      <c r="C22" s="9">
+        <v>420</v>
+      </c>
+      <c r="D22" s="9">
+        <v>25</v>
+      </c>
+      <c r="E22" s="9">
+        <v>35</v>
+      </c>
+      <c r="F22" s="9">
+        <v>45</v>
+      </c>
+      <c r="G22" s="9">
+        <v>360</v>
+      </c>
+      <c r="H22" s="9">
+        <v>6</v>
+      </c>
+      <c r="I22" s="9">
+        <v>90</v>
+      </c>
+      <c r="J22" s="10">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="K22" s="10" t="str">
+        <v>975</v>
+      </c>
+      <c r="K22" s="10">
         <f t="shared" si="3"/>
-        <v/>
-      </c>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="12"/>
+        <v>465</v>
+      </c>
+      <c r="L22" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="M22" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="N22" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="O22" s="12" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="str">

</xml_diff>